<commit_message>
Fix cashflow: 8360 paid in full (balance 0), zip-repair + kopeck tolerance
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Графік надходжень'!$A$1:$I$62</definedName>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Прострочені!$A$1:$G$5</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">Прострочені!$A$1:$G$4</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="73">
   <si>
     <t xml:space="preserve">Грошовий потік — звіт Pillar</t>
   </si>
@@ -816,7 +816,7 @@
       </c>
       <c r="B8" s="4" t="n">
         <f aca="false">SUMIF(Прострочені!A:A,"&lt;&gt;",Прострочені!G:G)</f>
-        <v>12322066.7</v>
+        <v>12322035</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1932,11 +1932,11 @@
         <v>95968.3</v>
       </c>
       <c r="G33" s="10" t="n">
-        <v>96000</v>
+        <v>95968.3</v>
       </c>
       <c r="H33" s="11" t="n">
         <f aca="false">F33-G33</f>
-        <v>-31.6999999999971</v>
+        <v>0</v>
       </c>
       <c r="I33" s="9" t="s">
         <v>25</v>
@@ -2196,14 +2196,14 @@
         <v>95968.3</v>
       </c>
       <c r="G41" s="10" t="n">
-        <v>95936.6</v>
+        <v>95968.3</v>
       </c>
       <c r="H41" s="11" t="n">
         <f aca="false">F41-G41</f>
-        <v>31.6999999999971</v>
+        <v>0</v>
       </c>
       <c r="I41" s="9" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J41" s="0" t="s">
         <v>51</v>
@@ -3125,7 +3125,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -3231,48 +3231,24 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="n">
-        <v>46197</v>
-      </c>
-      <c r="B5" s="9" t="n">
-        <v>8360</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>95968.3</v>
-      </c>
-      <c r="F5" s="11" t="n">
-        <v>95936.6</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <f aca="false">E5-F5</f>
-        <v>31.6999999999971</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="D6" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="E6" s="12" t="n">
-        <f aca="false">SUM(E2:E5)</f>
-        <v>14110041.3</v>
-      </c>
-      <c r="F6" s="12" t="n">
-        <f aca="false">SUM(F2:F5)</f>
-        <v>1787974.6</v>
-      </c>
-      <c r="G6" s="12" t="n">
-        <f aca="false">SUM(G2:G5)</f>
-        <v>12322066.7</v>
+      <c r="E5" s="12" t="n">
+        <f aca="false">SUM(E2:E4)</f>
+        <v>14014073</v>
+      </c>
+      <c r="F5" s="12" t="n">
+        <f aca="false">SUM(F2:F4)</f>
+        <v>1692038</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <f aca="false">SUM(G2:G4)</f>
+        <v>12322035</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G5"/>
+  <autoFilter ref="A1:G4"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Update 13.07.2026: Zayanchkovskyi re-export (overdue 10 -> 0)
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прострочені" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$65</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J66"/>
+  <dimension ref="A1:J68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2474,19 +2474,19 @@
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
-        <v>46206</v>
+        <v>46209</v>
       </c>
       <c r="B44" s="9" t="n">
-        <v>4766</v>
+        <v>8188</v>
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>Фундамент Ужгород Стефанія</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Александров</t>
         </is>
       </c>
       <c r="E44" s="9" t="inlineStr">
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="F44" s="10" t="n">
-        <v>100000</v>
+        <v>73926</v>
       </c>
       <c r="G44" s="10" t="n">
         <v>0</v>
@@ -2520,28 +2520,28 @@
         <v>46209</v>
       </c>
       <c r="B45" s="9" t="n">
-        <v>8188</v>
+        <v>8878</v>
       </c>
       <c r="C45" s="9" t="inlineStr">
         <is>
-          <t>Фундамент Ужгород Стефанія</t>
+          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
         </is>
       </c>
       <c r="D45" s="9" t="inlineStr">
         <is>
-          <t>Александров</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E45" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F45" s="10" t="n">
-        <v>73926</v>
+        <v>410320</v>
       </c>
       <c r="G45" s="10" t="n">
-        <v>0</v>
+        <v>410320</v>
       </c>
       <c r="H45" s="11">
         <f>F45-G45</f>
@@ -2549,7 +2549,7 @@
       </c>
       <c r="I45" s="9" t="inlineStr">
         <is>
-          <t>прострочено</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
@@ -2818,28 +2818,28 @@
     </row>
     <row r="52">
       <c r="A52" s="8" t="n">
-        <v>46225</v>
+        <v>46217</v>
       </c>
       <c r="B52" s="9" t="n">
-        <v>3456</v>
+        <v>4766</v>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>А Підселання фундаменту</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F52" s="10" t="n">
-        <v>335974.68</v>
+        <v>100000</v>
       </c>
       <c r="G52" s="10" t="n">
         <v>0</v>
@@ -2864,11 +2864,11 @@
         <v>46225</v>
       </c>
       <c r="B53" s="9" t="n">
-        <v>8008</v>
+        <v>3456</v>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>Модулі Григорівка</t>
+          <t>А Підселання фундаменту</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
@@ -2878,14 +2878,14 @@
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F53" s="10" t="n">
-        <v>178088.4</v>
+        <v>335974.68</v>
       </c>
       <c r="G53" s="10" t="n">
-        <v>178088.4</v>
+        <v>0</v>
       </c>
       <c r="H53" s="11">
         <f>F53-G53</f>
@@ -2893,7 +2893,7 @@
       </c>
       <c r="I53" s="9" t="inlineStr">
         <is>
-          <t>отримано</t>
+          <t>очікується</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -2904,14 +2904,14 @@
     </row>
     <row r="54">
       <c r="A54" s="8" t="n">
-        <v>46228</v>
+        <v>46225</v>
       </c>
       <c r="B54" s="9" t="n">
-        <v>5910</v>
+        <v>8008</v>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>А   AGM 2V</t>
+          <t>Модулі Григорівка</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
@@ -2925,10 +2925,10 @@
         </is>
       </c>
       <c r="F54" s="10" t="n">
-        <v>17035932.8</v>
+        <v>178088.4</v>
       </c>
       <c r="G54" s="10" t="n">
-        <v>0</v>
+        <v>178088.4</v>
       </c>
       <c r="H54" s="11">
         <f>F54-G54</f>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="I54" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2947,14 +2947,14 @@
     </row>
     <row r="55">
       <c r="A55" s="8" t="n">
-        <v>46231</v>
+        <v>46228</v>
       </c>
       <c r="B55" s="9" t="n">
-        <v>7894</v>
+        <v>5910</v>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>А   AGM 2V</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -2964,11 +2964,11 @@
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F55" s="10" t="n">
-        <v>737597.4</v>
+        <v>17035932.8</v>
       </c>
       <c r="G55" s="10" t="n">
         <v>0</v>
@@ -2990,14 +2990,14 @@
     </row>
     <row r="56">
       <c r="A56" s="8" t="n">
-        <v>46233</v>
+        <v>46231</v>
       </c>
       <c r="B56" s="9" t="n">
-        <v>8008</v>
+        <v>7894</v>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>Модулі Григорівка</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
@@ -3007,11 +3007,11 @@
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F56" s="10" t="n">
-        <v>178088.4</v>
+        <v>737597.4</v>
       </c>
       <c r="G56" s="10" t="n">
         <v>0</v>
@@ -3033,19 +3033,19 @@
     </row>
     <row r="57">
       <c r="A57" s="8" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="B57" s="9" t="n">
-        <v>7068</v>
+        <v>8008</v>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>А Remtec energy  AGM  160 TP</t>
+          <t>Модулі Григорівка</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Александров</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
@@ -3054,10 +3054,10 @@
         </is>
       </c>
       <c r="F57" s="10" t="n">
+        <v>178088.4</v>
+      </c>
+      <c r="G57" s="10" t="n">
         <v>0</v>
-      </c>
-      <c r="G57" s="10" t="n">
-        <v>2794670</v>
       </c>
       <c r="H57" s="11">
         <f>F57-G57</f>
@@ -3079,28 +3079,28 @@
         <v>46234</v>
       </c>
       <c r="B58" s="9" t="n">
-        <v>7244</v>
+        <v>7068</v>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>В Модулекс модульна будівля Чернігів</t>
+          <t>А Remtec energy  AGM  160 TP</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Александров</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F58" s="10" t="n">
-        <v>132708.6</v>
+        <v>0</v>
       </c>
       <c r="G58" s="10" t="n">
-        <v>0</v>
+        <v>2794670</v>
       </c>
       <c r="H58" s="11">
         <f>F58-G58</f>
@@ -3122,25 +3122,25 @@
         <v>46234</v>
       </c>
       <c r="B59" s="9" t="n">
-        <v>7894</v>
+        <v>7244</v>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>В Модулекс модульна будівля Чернігів</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F59" s="10" t="n">
-        <v>185968</v>
+        <v>132708.6</v>
       </c>
       <c r="G59" s="10" t="n">
         <v>0</v>
@@ -3162,7 +3162,7 @@
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
-        <v>46245</v>
+        <v>46234</v>
       </c>
       <c r="B60" s="9" t="n">
         <v>7894</v>
@@ -3179,11 +3179,11 @@
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F60" s="10" t="n">
-        <v>185967.99</v>
+        <v>185968</v>
       </c>
       <c r="G60" s="10" t="n">
         <v>0</v>
@@ -3199,34 +3199,34 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n">
-        <v>46249</v>
+        <v>46237</v>
       </c>
       <c r="B61" s="9" t="n">
-        <v>7002</v>
+        <v>8878</v>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP W 24PS V1</t>
+          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F61" s="10" t="n">
-        <v>573945</v>
+        <v>12823</v>
       </c>
       <c r="G61" s="10" t="n">
         <v>0</v>
@@ -3248,14 +3248,14 @@
     </row>
     <row r="62">
       <c r="A62" s="8" t="n">
-        <v>46260</v>
+        <v>46245</v>
       </c>
       <c r="B62" s="9" t="n">
-        <v>5910</v>
+        <v>7894</v>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>А   AGM 2V</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
@@ -3269,7 +3269,7 @@
         </is>
       </c>
       <c r="F62" s="10" t="n">
-        <v>2896238.8</v>
+        <v>185967.99</v>
       </c>
       <c r="G62" s="10" t="n">
         <v>0</v>
@@ -3291,7 +3291,7 @@
     </row>
     <row r="63">
       <c r="A63" s="8" t="n">
-        <v>46260</v>
+        <v>46249</v>
       </c>
       <c r="B63" s="9" t="n">
         <v>7002</v>
@@ -3308,7 +3308,7 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F63" s="10" t="n">
@@ -3334,14 +3334,14 @@
     </row>
     <row r="64">
       <c r="A64" s="8" t="n">
-        <v>46282</v>
+        <v>46260</v>
       </c>
       <c r="B64" s="9" t="n">
-        <v>7894</v>
+        <v>5910</v>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>А   AGM 2V</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -3351,11 +3351,11 @@
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F64" s="10" t="n">
-        <v>737597.4</v>
+        <v>2896238.8</v>
       </c>
       <c r="G64" s="10" t="n">
         <v>0</v>
@@ -3371,25 +3371,25 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n">
-        <v>46287</v>
+        <v>46260</v>
       </c>
       <c r="B65" s="9" t="n">
-        <v>4766</v>
+        <v>7002</v>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>А Фора  SCP W 24PS V1</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
@@ -3398,7 +3398,7 @@
         </is>
       </c>
       <c r="F65" s="10" t="n">
-        <v>4880000</v>
+        <v>573945</v>
       </c>
       <c r="G65" s="10" t="n">
         <v>0</v>
@@ -3414,31 +3414,117 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B66" s="9" t="n">
+        <v>7894</v>
+      </c>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>А Фора  SCP  32PS</t>
+        </is>
+      </c>
+      <c r="D66" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E66" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F66" s="10" t="n">
+        <v>737597.4</v>
+      </c>
+      <c r="G66" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" s="11">
+        <f>F66-G66</f>
+        <v/>
+      </c>
+      <c r="I66" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
           <t>2026-09</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="E66" s="3" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="8" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B67" s="9" t="n">
+        <v>4766</v>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
+        </is>
+      </c>
+      <c r="D67" s="9" t="inlineStr">
+        <is>
+          <t>Заянчковський</t>
+        </is>
+      </c>
+      <c r="E67" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F67" s="10" t="n">
+        <v>4880000</v>
+      </c>
+      <c r="G67" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" s="11">
+        <f>F67-G67</f>
+        <v/>
+      </c>
+      <c r="I67" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="E68" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="F66" s="12">
-        <f>SUM(F2:F65)</f>
-        <v/>
-      </c>
-      <c r="G66" s="12">
-        <f>SUM(G2:G65)</f>
-        <v/>
-      </c>
-      <c r="H66" s="12">
-        <f>SUM(H2:H65)</f>
+      <c r="F68" s="12">
+        <f>SUM(F2:F67)</f>
+        <v/>
+      </c>
+      <c r="G68" s="12">
+        <f>SUM(G2:G67)</f>
+        <v/>
+      </c>
+      <c r="H68" s="12">
+        <f>SUM(H2:H67)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I65"/>
+  <autoFilter ref="A1:I67"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3658,7 +3744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3905,14 +3991,14 @@
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
-        <v>46206</v>
+        <v>46209</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>4766</v>
+        <v>8188</v>
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>Фундамент Ужгород Стефанія</t>
         </is>
       </c>
       <c r="D9" s="9" t="inlineStr">
@@ -3921,7 +4007,7 @@
         </is>
       </c>
       <c r="E9" s="11" t="n">
-        <v>100000</v>
+        <v>73926</v>
       </c>
       <c r="F9" s="11" t="n">
         <v>0</v>
@@ -3933,14 +4019,14 @@
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
-        <v>46209</v>
+        <v>46213</v>
       </c>
       <c r="B10" s="9" t="n">
-        <v>8188</v>
+        <v>8185</v>
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
-          <t>Фундамент Ужгород Стефанія</t>
+          <t>Фундамент Hytte House Development Славське</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -3949,7 +4035,7 @@
         </is>
       </c>
       <c r="E10" s="11" t="n">
-        <v>73926</v>
+        <v>63313.4</v>
       </c>
       <c r="F10" s="11" t="n">
         <v>0</v>
@@ -3973,7 +4059,7 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="E11" s="11" t="n">
@@ -3988,54 +4074,26 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="n">
-        <v>46213</v>
-      </c>
-      <c r="B12" s="9" t="n">
-        <v>8185</v>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Фундамент Hytte House Development Славське</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Третій платіж</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>63313.4</v>
-      </c>
-      <c r="F12" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="11">
-        <f>E12-F12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="E13" s="12">
-        <f>SUM(E2:E12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="12">
-        <f>SUM(F2:F12)</f>
-        <v/>
-      </c>
-      <c r="G13" s="12">
-        <f>SUM(G2:G12)</f>
+      <c r="E12" s="12">
+        <f>SUM(E2:E11)</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>SUM(F2:F11)</f>
+        <v/>
+      </c>
+      <c r="G12" s="12">
+        <f>SUM(G2:G11)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G12"/>
+  <autoFilter ref="A1:G11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Multi-currency: 8496 EUR budget, NBU rate conversion (EUR 50.86)
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прострочені" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$67</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$68</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -599,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J68"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2818,31 +2818,31 @@
     </row>
     <row r="52">
       <c r="A52" s="8" t="n">
-        <v>46217</v>
+        <v>46216</v>
       </c>
       <c r="B52" s="9" t="n">
-        <v>4766</v>
+        <v>8496</v>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>А Greensource  SGM  110MWp</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Іщук</t>
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Авансовий платіж (€8 800)</t>
         </is>
       </c>
       <c r="F52" s="10" t="n">
-        <v>100000</v>
+        <v>447568</v>
       </c>
       <c r="G52" s="10" t="n">
-        <v>0</v>
+        <v>447568</v>
       </c>
       <c r="H52" s="11">
         <f>F52-G52</f>
@@ -2850,7 +2850,7 @@
       </c>
       <c r="I52" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
@@ -2861,28 +2861,28 @@
     </row>
     <row r="53">
       <c r="A53" s="8" t="n">
-        <v>46225</v>
+        <v>46217</v>
       </c>
       <c r="B53" s="9" t="n">
-        <v>3456</v>
+        <v>4766</v>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>А Підселання фундаменту</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F53" s="10" t="n">
-        <v>335974.68</v>
+        <v>100000</v>
       </c>
       <c r="G53" s="10" t="n">
         <v>0</v>
@@ -2907,11 +2907,11 @@
         <v>46225</v>
       </c>
       <c r="B54" s="9" t="n">
-        <v>8008</v>
+        <v>3456</v>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>Модулі Григорівка</t>
+          <t>А Підселання фундаменту</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
@@ -2921,14 +2921,14 @@
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F54" s="10" t="n">
-        <v>178088.4</v>
+        <v>335974.68</v>
       </c>
       <c r="G54" s="10" t="n">
-        <v>178088.4</v>
+        <v>0</v>
       </c>
       <c r="H54" s="11">
         <f>F54-G54</f>
@@ -2936,7 +2936,7 @@
       </c>
       <c r="I54" s="9" t="inlineStr">
         <is>
-          <t>отримано</t>
+          <t>очікується</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -2947,14 +2947,14 @@
     </row>
     <row r="55">
       <c r="A55" s="8" t="n">
-        <v>46228</v>
+        <v>46225</v>
       </c>
       <c r="B55" s="9" t="n">
-        <v>5910</v>
+        <v>8008</v>
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>А   AGM 2V</t>
+          <t>Модулі Григорівка</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -2968,10 +2968,10 @@
         </is>
       </c>
       <c r="F55" s="10" t="n">
-        <v>17035932.8</v>
+        <v>178088.4</v>
       </c>
       <c r="G55" s="10" t="n">
-        <v>0</v>
+        <v>178088.4</v>
       </c>
       <c r="H55" s="11">
         <f>F55-G55</f>
@@ -2979,7 +2979,7 @@
       </c>
       <c r="I55" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
@@ -2990,14 +2990,14 @@
     </row>
     <row r="56">
       <c r="A56" s="8" t="n">
-        <v>46231</v>
+        <v>46228</v>
       </c>
       <c r="B56" s="9" t="n">
-        <v>7894</v>
+        <v>5910</v>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>А   AGM 2V</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
@@ -3007,11 +3007,11 @@
       </c>
       <c r="E56" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F56" s="10" t="n">
-        <v>737597.4</v>
+        <v>17035932.8</v>
       </c>
       <c r="G56" s="10" t="n">
         <v>0</v>
@@ -3033,14 +3033,14 @@
     </row>
     <row r="57">
       <c r="A57" s="8" t="n">
-        <v>46233</v>
+        <v>46231</v>
       </c>
       <c r="B57" s="9" t="n">
-        <v>8008</v>
+        <v>7894</v>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Модулі Григорівка</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
@@ -3050,11 +3050,11 @@
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F57" s="10" t="n">
-        <v>178088.4</v>
+        <v>737597.4</v>
       </c>
       <c r="G57" s="10" t="n">
         <v>0</v>
@@ -3076,19 +3076,19 @@
     </row>
     <row r="58">
       <c r="A58" s="8" t="n">
-        <v>46234</v>
+        <v>46233</v>
       </c>
       <c r="B58" s="9" t="n">
-        <v>7068</v>
+        <v>8008</v>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>А Remtec energy  AGM  160 TP</t>
+          <t>Модулі Григорівка</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Александров</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
@@ -3097,10 +3097,10 @@
         </is>
       </c>
       <c r="F58" s="10" t="n">
+        <v>178088.4</v>
+      </c>
+      <c r="G58" s="10" t="n">
         <v>0</v>
-      </c>
-      <c r="G58" s="10" t="n">
-        <v>2794670</v>
       </c>
       <c r="H58" s="11">
         <f>F58-G58</f>
@@ -3122,28 +3122,28 @@
         <v>46234</v>
       </c>
       <c r="B59" s="9" t="n">
-        <v>7244</v>
+        <v>7068</v>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>В Модулекс модульна будівля Чернігів</t>
+          <t>А Remtec energy  AGM  160 TP</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Александров</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F59" s="10" t="n">
-        <v>132708.6</v>
+        <v>0</v>
       </c>
       <c r="G59" s="10" t="n">
-        <v>0</v>
+        <v>2794670</v>
       </c>
       <c r="H59" s="11">
         <f>F59-G59</f>
@@ -3165,25 +3165,25 @@
         <v>46234</v>
       </c>
       <c r="B60" s="9" t="n">
-        <v>7894</v>
+        <v>7244</v>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>В Модулекс модульна будівля Чернігів</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F60" s="10" t="n">
-        <v>185968</v>
+        <v>132708.6</v>
       </c>
       <c r="G60" s="10" t="n">
         <v>0</v>
@@ -3205,28 +3205,28 @@
     </row>
     <row r="61">
       <c r="A61" s="8" t="n">
-        <v>46237</v>
+        <v>46234</v>
       </c>
       <c r="B61" s="9" t="n">
-        <v>8878</v>
+        <v>7894</v>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F61" s="10" t="n">
-        <v>12823</v>
+        <v>185968</v>
       </c>
       <c r="G61" s="10" t="n">
         <v>0</v>
@@ -3242,34 +3242,34 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="B62" s="9" t="n">
-        <v>7894</v>
+        <v>8878</v>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F62" s="10" t="n">
-        <v>185967.99</v>
+        <v>12823</v>
       </c>
       <c r="G62" s="10" t="n">
         <v>0</v>
@@ -3291,14 +3291,14 @@
     </row>
     <row r="63">
       <c r="A63" s="8" t="n">
-        <v>46249</v>
+        <v>46245</v>
       </c>
       <c r="B63" s="9" t="n">
-        <v>7002</v>
+        <v>7894</v>
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP W 24PS V1</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -3308,11 +3308,11 @@
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F63" s="10" t="n">
-        <v>573945</v>
+        <v>185967.99</v>
       </c>
       <c r="G63" s="10" t="n">
         <v>0</v>
@@ -3334,14 +3334,14 @@
     </row>
     <row r="64">
       <c r="A64" s="8" t="n">
-        <v>46260</v>
+        <v>46249</v>
       </c>
       <c r="B64" s="9" t="n">
-        <v>5910</v>
+        <v>7002</v>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>А   AGM 2V</t>
+          <t>А Фора  SCP W 24PS V1</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -3351,11 +3351,11 @@
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F64" s="10" t="n">
-        <v>2896238.8</v>
+        <v>573945</v>
       </c>
       <c r="G64" s="10" t="n">
         <v>0</v>
@@ -3380,11 +3380,11 @@
         <v>46260</v>
       </c>
       <c r="B65" s="9" t="n">
-        <v>7002</v>
+        <v>5910</v>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP W 24PS V1</t>
+          <t>А   AGM 2V</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -3394,11 +3394,11 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F65" s="10" t="n">
-        <v>573945</v>
+        <v>2896238.8</v>
       </c>
       <c r="G65" s="10" t="n">
         <v>0</v>
@@ -3420,14 +3420,14 @@
     </row>
     <row r="66">
       <c r="A66" s="8" t="n">
-        <v>46282</v>
+        <v>46260</v>
       </c>
       <c r="B66" s="9" t="n">
-        <v>7894</v>
+        <v>7002</v>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>А Фора  SCP W 24PS V1</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
@@ -3441,7 +3441,7 @@
         </is>
       </c>
       <c r="F66" s="10" t="n">
-        <v>737597.4</v>
+        <v>573945</v>
       </c>
       <c r="G66" s="10" t="n">
         <v>0</v>
@@ -3457,25 +3457,25 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n">
-        <v>46287</v>
+        <v>46282</v>
       </c>
       <c r="B67" s="9" t="n">
-        <v>4766</v>
+        <v>7894</v>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
@@ -3484,7 +3484,7 @@
         </is>
       </c>
       <c r="F67" s="10" t="n">
-        <v>4880000</v>
+        <v>737597.4</v>
       </c>
       <c r="G67" s="10" t="n">
         <v>0</v>
@@ -3505,26 +3505,69 @@
       </c>
     </row>
     <row r="68">
-      <c r="E68" s="3" t="inlineStr">
+      <c r="A68" s="8" t="n">
+        <v>46287</v>
+      </c>
+      <c r="B68" s="9" t="n">
+        <v>4766</v>
+      </c>
+      <c r="C68" s="9" t="inlineStr">
+        <is>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
+        </is>
+      </c>
+      <c r="D68" s="9" t="inlineStr">
+        <is>
+          <t>Заянчковський</t>
+        </is>
+      </c>
+      <c r="E68" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F68" s="10" t="n">
+        <v>4880000</v>
+      </c>
+      <c r="G68" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" s="11">
+        <f>F68-G68</f>
+        <v/>
+      </c>
+      <c r="I68" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="E69" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="F68" s="12">
-        <f>SUM(F2:F67)</f>
-        <v/>
-      </c>
-      <c r="G68" s="12">
-        <f>SUM(G2:G67)</f>
-        <v/>
-      </c>
-      <c r="H68" s="12">
-        <f>SUM(H2:H67)</f>
+      <c r="F69" s="12">
+        <f>SUM(F2:F68)</f>
+        <v/>
+      </c>
+      <c r="G69" s="12">
+        <f>SUM(G2:G68)</f>
+        <v/>
+      </c>
+      <c r="H69" s="12">
+        <f>SUM(H2:H68)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I67"/>
+  <autoFilter ref="A1:I68"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Currency toggle UAH/EUR on KPIs + native currency column in cashflow
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -133,6 +133,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -599,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J69"/>
+  <dimension ref="A1:K69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -612,6 +613,7 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col hidden="1" width="9" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -665,6 +667,11 @@
           <t>YM</t>
         </is>
       </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>У валюті</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="n">
@@ -708,6 +715,7 @@
           <t>2026-04</t>
         </is>
       </c>
+      <c r="K2" s="12" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="8" t="n">
@@ -751,6 +759,7 @@
           <t>2026-04</t>
         </is>
       </c>
+      <c r="K3" s="12" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
@@ -794,6 +803,7 @@
           <t>2026-04</t>
         </is>
       </c>
+      <c r="K4" s="12" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="n">
@@ -837,6 +847,7 @@
           <t>2026-04</t>
         </is>
       </c>
+      <c r="K5" s="12" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
@@ -880,6 +891,7 @@
           <t>2026-04</t>
         </is>
       </c>
+      <c r="K6" s="12" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n">
@@ -923,6 +935,7 @@
           <t>2026-04</t>
         </is>
       </c>
+      <c r="K7" s="12" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n">
@@ -966,6 +979,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K8" s="12" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n">
@@ -1009,6 +1023,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K9" s="12" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n">
@@ -1052,6 +1067,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K10" s="12" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n">
@@ -1095,6 +1111,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K11" s="12" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
@@ -1138,6 +1155,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K12" s="12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n">
@@ -1181,6 +1199,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K13" s="12" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
@@ -1224,6 +1243,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K14" s="12" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n">
@@ -1267,6 +1287,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K15" s="12" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n">
@@ -1310,6 +1331,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K16" s="12" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n">
@@ -1353,6 +1375,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K17" s="12" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n">
@@ -1396,6 +1419,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K18" s="12" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n">
@@ -1439,6 +1463,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K19" s="12" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
@@ -1482,6 +1507,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K20" s="12" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n">
@@ -1525,6 +1551,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K21" s="12" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n">
@@ -1568,6 +1595,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K22" s="12" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n">
@@ -1611,6 +1639,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K23" s="12" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n">
@@ -1654,6 +1683,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K24" s="12" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n">
@@ -1697,6 +1727,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K25" s="12" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n">
@@ -1740,6 +1771,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K26" s="12" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="n">
@@ -1783,6 +1815,7 @@
           <t>2026-05</t>
         </is>
       </c>
+      <c r="K27" s="12" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n">
@@ -1826,6 +1859,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K28" s="12" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n">
@@ -1869,6 +1903,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K29" s="12" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n">
@@ -1912,6 +1947,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K30" s="12" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n">
@@ -1955,6 +1991,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K31" s="12" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n">
@@ -1998,6 +2035,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K32" s="12" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n">
@@ -2041,6 +2079,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K33" s="12" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n">
@@ -2084,6 +2123,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K34" s="12" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n">
@@ -2127,6 +2167,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K35" s="12" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n">
@@ -2170,6 +2211,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K36" s="12" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n">
@@ -2213,6 +2255,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K37" s="12" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n">
@@ -2256,6 +2299,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K38" s="12" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n">
@@ -2299,6 +2343,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K39" s="12" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n">
@@ -2342,6 +2387,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K40" s="12" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n">
@@ -2385,6 +2431,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K41" s="12" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n">
@@ -2428,6 +2475,7 @@
           <t>2026-06</t>
         </is>
       </c>
+      <c r="K42" s="12" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n">
@@ -2471,6 +2519,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K43" s="12" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
@@ -2514,6 +2563,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K44" s="12" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="n">
@@ -2557,6 +2607,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K45" s="12" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n">
@@ -2600,6 +2651,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K46" s="12" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="n">
@@ -2643,6 +2695,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K47" s="12" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n">
@@ -2686,6 +2739,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K48" s="12" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n">
@@ -2729,6 +2783,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K49" s="12" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n">
@@ -2772,6 +2827,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K50" s="12" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="n">
@@ -2815,6 +2871,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K51" s="12" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n">
@@ -2835,7 +2892,7 @@
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Авансовий платіж (€8 800)</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F52" s="10" t="n">
@@ -2856,6 +2913,11 @@
       <c r="J52" t="inlineStr">
         <is>
           <t>2026-07</t>
+        </is>
+      </c>
+      <c r="K52" s="12" t="inlineStr">
+        <is>
+          <t>€8 800</t>
         </is>
       </c>
     </row>
@@ -2901,6 +2963,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K53" s="12" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="8" t="n">
@@ -2944,6 +3007,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K54" s="12" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n">
@@ -2987,6 +3051,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K55" s="12" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="8" t="n">
@@ -3030,6 +3095,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K56" s="12" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="8" t="n">
@@ -3073,6 +3139,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K57" s="12" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="n">
@@ -3116,6 +3183,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K58" s="12" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n">
@@ -3159,6 +3227,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K59" s="12" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
@@ -3202,6 +3271,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K60" s="12" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n">
@@ -3245,6 +3315,7 @@
           <t>2026-07</t>
         </is>
       </c>
+      <c r="K61" s="12" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n">
@@ -3288,6 +3359,7 @@
           <t>2026-08</t>
         </is>
       </c>
+      <c r="K62" s="12" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n">
@@ -3331,6 +3403,7 @@
           <t>2026-08</t>
         </is>
       </c>
+      <c r="K63" s="12" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="8" t="n">
@@ -3374,6 +3447,7 @@
           <t>2026-08</t>
         </is>
       </c>
+      <c r="K64" s="12" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n">
@@ -3417,6 +3491,7 @@
           <t>2026-08</t>
         </is>
       </c>
+      <c r="K65" s="12" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="8" t="n">
@@ -3460,6 +3535,7 @@
           <t>2026-08</t>
         </is>
       </c>
+      <c r="K66" s="12" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n">
@@ -3503,6 +3579,7 @@
           <t>2026-09</t>
         </is>
       </c>
+      <c r="K67" s="12" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
@@ -3546,6 +3623,7 @@
           <t>2026-09</t>
         </is>
       </c>
+      <c r="K68" s="12" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="E69" s="3" t="inlineStr">
@@ -3553,15 +3631,15 @@
           <t>Разом</t>
         </is>
       </c>
-      <c r="F69" s="12">
+      <c r="F69" s="13">
         <f>SUM(F2:F68)</f>
         <v/>
       </c>
-      <c r="G69" s="12">
+      <c r="G69" s="13">
         <f>SUM(G2:G68)</f>
         <v/>
       </c>
-      <c r="H69" s="12">
+      <c r="H69" s="13">
         <f>SUM(H2:H68)</f>
         <v/>
       </c>
@@ -3633,7 +3711,7 @@
         <f>B2-C2</f>
         <v/>
       </c>
-      <c r="E2" s="13">
+      <c r="E2" s="14">
         <f>IF(B2=0,0,C2/B2)</f>
         <v/>
       </c>
@@ -3656,7 +3734,7 @@
         <f>B3-C3</f>
         <v/>
       </c>
-      <c r="E3" s="13">
+      <c r="E3" s="14">
         <f>IF(B3=0,0,C3/B3)</f>
         <v/>
       </c>
@@ -3679,7 +3757,7 @@
         <f>B4-C4</f>
         <v/>
       </c>
-      <c r="E4" s="13">
+      <c r="E4" s="14">
         <f>IF(B4=0,0,C4/B4)</f>
         <v/>
       </c>
@@ -3702,7 +3780,7 @@
         <f>B5-C5</f>
         <v/>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="14">
         <f>IF(B5=0,0,C5/B5)</f>
         <v/>
       </c>
@@ -3725,7 +3803,7 @@
         <f>B6-C6</f>
         <v/>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="14">
         <f>IF(B6=0,0,C6/B6)</f>
         <v/>
       </c>
@@ -3748,7 +3826,7 @@
         <f>B7-C7</f>
         <v/>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="14">
         <f>IF(B7=0,0,C7/B7)</f>
         <v/>
       </c>
@@ -3759,19 +3837,19 @@
           <t>Разом</t>
         </is>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="13">
         <f>SUM(B2:B7)</f>
         <v/>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="13">
         <f>SUM(C2:C7)</f>
         <v/>
       </c>
-      <c r="D8" s="12">
+      <c r="D8" s="13">
         <f>SUM(D2:D7)</f>
         <v/>
       </c>
-      <c r="E8" s="14">
+      <c r="E8" s="15">
         <f>IF(B8=0,0,C8/B8)</f>
         <v/>
       </c>
@@ -4122,15 +4200,15 @@
           <t>Разом</t>
         </is>
       </c>
-      <c r="E12" s="12">
+      <c r="E12" s="13">
         <f>SUM(E2:E11)</f>
         <v/>
       </c>
-      <c r="F12" s="12">
+      <c r="F12" s="13">
         <f>SUM(F2:F11)</f>
         <v/>
       </c>
-      <c r="G12" s="12">
+      <c r="G12" s="13">
         <f>SUM(G2:G11)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Fix 4766: uninactivate 3rd+4th payments (budget labels removed)
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прострочені" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$69</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$71</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K70"/>
+  <dimension ref="A1:K72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3191,28 +3191,28 @@
     </row>
     <row r="59">
       <c r="A59" s="8" t="n">
-        <v>46231</v>
+        <v>46227</v>
       </c>
       <c r="B59" s="9" t="n">
-        <v>7894</v>
+        <v>4766</v>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F59" s="10" t="n">
-        <v>737597.4</v>
+        <v>4368478.98</v>
       </c>
       <c r="G59" s="10" t="n">
         <v>0</v>
@@ -3235,31 +3235,31 @@
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
-        <v>46234</v>
+        <v>46231</v>
       </c>
       <c r="B60" s="9" t="n">
-        <v>7068</v>
+        <v>7894</v>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>А Remtec energy  AGM  160 TP</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Александров</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F60" s="10" t="n">
+        <v>737597.4</v>
+      </c>
+      <c r="G60" s="10" t="n">
         <v>0</v>
-      </c>
-      <c r="G60" s="10" t="n">
-        <v>2794670</v>
       </c>
       <c r="H60" s="11">
         <f>F60-G60</f>
@@ -3282,28 +3282,28 @@
         <v>46234</v>
       </c>
       <c r="B61" s="9" t="n">
-        <v>7244</v>
+        <v>7068</v>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>В Модулекс модульна будівля Чернігів</t>
+          <t>А Remtec energy  AGM  160 TP</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Александров</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F61" s="10" t="n">
-        <v>132708.6</v>
+        <v>0</v>
       </c>
       <c r="G61" s="10" t="n">
-        <v>0</v>
+        <v>2794670</v>
       </c>
       <c r="H61" s="11">
         <f>F61-G61</f>
@@ -3323,28 +3323,28 @@
     </row>
     <row r="62">
       <c r="A62" s="8" t="n">
-        <v>46237</v>
+        <v>46234</v>
       </c>
       <c r="B62" s="9" t="n">
-        <v>7894</v>
+        <v>7244</v>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>В Модулекс модульна будівля Чернігів</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F62" s="10" t="n">
-        <v>185968</v>
+        <v>132708.6</v>
       </c>
       <c r="G62" s="10" t="n">
         <v>0</v>
@@ -3360,7 +3360,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="K62" s="12" t="inlineStr"/>
@@ -3370,25 +3370,25 @@
         <v>46237</v>
       </c>
       <c r="B63" s="9" t="n">
-        <v>8878</v>
+        <v>7894</v>
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F63" s="10" t="n">
-        <v>12823</v>
+        <v>185968</v>
       </c>
       <c r="G63" s="10" t="n">
         <v>0</v>
@@ -3411,28 +3411,28 @@
     </row>
     <row r="64">
       <c r="A64" s="8" t="n">
-        <v>46239</v>
+        <v>46237</v>
       </c>
       <c r="B64" s="9" t="n">
-        <v>5910</v>
+        <v>8878</v>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>А   AGM 2V</t>
+          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E64" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F64" s="10" t="n">
-        <v>17073327.726</v>
+        <v>12823</v>
       </c>
       <c r="G64" s="10" t="n">
         <v>0</v>
@@ -3451,22 +3451,18 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K64" s="12" t="inlineStr">
-        <is>
-          <t>€334 181</t>
-        </is>
-      </c>
+      <c r="K64" s="12" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n">
-        <v>46245</v>
+        <v>46239</v>
       </c>
       <c r="B65" s="9" t="n">
-        <v>7894</v>
+        <v>5910</v>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>А   AGM 2V</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -3476,11 +3472,11 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F65" s="10" t="n">
-        <v>185967.99</v>
+        <v>17073327.726</v>
       </c>
       <c r="G65" s="10" t="n">
         <v>0</v>
@@ -3499,18 +3495,22 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K65" s="12" t="inlineStr"/>
+      <c r="K65" s="12" t="inlineStr">
+        <is>
+          <t>€334 181</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="n">
-        <v>46260</v>
+        <v>46245</v>
       </c>
       <c r="B66" s="9" t="n">
-        <v>7002</v>
+        <v>7894</v>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP W 24PS V1</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
@@ -3520,11 +3520,11 @@
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F66" s="10" t="n">
-        <v>573945</v>
+        <v>185967.99</v>
       </c>
       <c r="G66" s="10" t="n">
         <v>0</v>
@@ -3547,19 +3547,19 @@
     </row>
     <row r="67">
       <c r="A67" s="8" t="n">
-        <v>46267</v>
+        <v>46260</v>
       </c>
       <c r="B67" s="9" t="n">
-        <v>4766</v>
+        <v>7002</v>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>А Фора  SCP W 24PS V1</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
@@ -3568,7 +3568,7 @@
         </is>
       </c>
       <c r="F67" s="10" t="n">
-        <v>1199397.42</v>
+        <v>573945</v>
       </c>
       <c r="G67" s="10" t="n">
         <v>0</v>
@@ -3584,35 +3584,35 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="K67" s="12" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
-        <v>46271</v>
+        <v>46266</v>
       </c>
       <c r="B68" s="9" t="n">
-        <v>5910</v>
+        <v>4766</v>
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>А   AGM 2V</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F68" s="10" t="n">
-        <v>2845554.621</v>
+        <v>128100</v>
       </c>
       <c r="G68" s="10" t="n">
         <v>0</v>
@@ -3631,27 +3631,23 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="K68" s="12" t="inlineStr">
-        <is>
-          <t>€55 697</t>
-        </is>
-      </c>
+      <c r="K68" s="12" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
-        <v>46282</v>
+        <v>46267</v>
       </c>
       <c r="B69" s="9" t="n">
-        <v>7894</v>
+        <v>4766</v>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
@@ -3660,7 +3656,7 @@
         </is>
       </c>
       <c r="F69" s="10" t="n">
-        <v>737597.4</v>
+        <v>1199397.42</v>
       </c>
       <c r="G69" s="10" t="n">
         <v>0</v>
@@ -3682,26 +3678,118 @@
       <c r="K69" s="12" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="E70" s="3" t="inlineStr">
+      <c r="A70" s="8" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B70" s="9" t="n">
+        <v>5910</v>
+      </c>
+      <c r="C70" s="9" t="inlineStr">
+        <is>
+          <t>А   AGM 2V</t>
+        </is>
+      </c>
+      <c r="D70" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E70" s="9" t="inlineStr">
+        <is>
+          <t>Третій платіж</t>
+        </is>
+      </c>
+      <c r="F70" s="10" t="n">
+        <v>2845554.621</v>
+      </c>
+      <c r="G70" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H70" s="11">
+        <f>F70-G70</f>
+        <v/>
+      </c>
+      <c r="I70" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K70" s="12" t="inlineStr">
+        <is>
+          <t>€55 697</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B71" s="9" t="n">
+        <v>7894</v>
+      </c>
+      <c r="C71" s="9" t="inlineStr">
+        <is>
+          <t>А Фора  SCP  32PS</t>
+        </is>
+      </c>
+      <c r="D71" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E71" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F71" s="10" t="n">
+        <v>737597.4</v>
+      </c>
+      <c r="G71" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" s="11">
+        <f>F71-G71</f>
+        <v/>
+      </c>
+      <c r="I71" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K71" s="12" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="E72" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="F70" s="13">
-        <f>SUM(F2:F69)</f>
-        <v/>
-      </c>
-      <c r="G70" s="13">
-        <f>SUM(G2:G69)</f>
-        <v/>
-      </c>
-      <c r="H70" s="13">
-        <f>SUM(H2:H69)</f>
+      <c r="F72" s="13">
+        <f>SUM(F2:F71)</f>
+        <v/>
+      </c>
+      <c r="G72" s="13">
+        <f>SUM(G2:G71)</f>
+        <v/>
+      </c>
+      <c r="H72" s="13">
+        <f>SUM(H2:H71)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I69"/>
+  <autoFilter ref="A1:I71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
5870 & 6704: manual UAH->EUR at 52 (temp until labeled export)
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -1136,10 +1136,10 @@
         </is>
       </c>
       <c r="F12" s="10" t="n">
-        <v>2600000</v>
+        <v>2553000</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>2600000</v>
+        <v>2553000</v>
       </c>
       <c r="H12" s="11">
         <f>F12-G12</f>
@@ -1155,7 +1155,11 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="K12" s="12" t="inlineStr"/>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>€50 000</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n">
@@ -1180,10 +1184,10 @@
         </is>
       </c>
       <c r="F13" s="10" t="n">
-        <v>5200000</v>
+        <v>5106000</v>
       </c>
       <c r="G13" s="10" t="n">
-        <v>5200000</v>
+        <v>5106000</v>
       </c>
       <c r="H13" s="11">
         <f>F13-G13</f>
@@ -1199,7 +1203,11 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="K13" s="12" t="inlineStr"/>
+      <c r="K13" s="12" t="inlineStr">
+        <is>
+          <t>€100 000</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n">
@@ -1444,7 +1452,7 @@
         </is>
       </c>
       <c r="F19" s="10" t="n">
-        <v>4524000</v>
+        <v>4442220</v>
       </c>
       <c r="G19" s="10" t="n">
         <v>0</v>
@@ -1463,7 +1471,11 @@
           <t>2026-05</t>
         </is>
       </c>
-      <c r="K19" s="12" t="inlineStr"/>
+      <c r="K19" s="12" t="inlineStr">
+        <is>
+          <t>€87 000</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n">
@@ -2456,10 +2468,10 @@
         </is>
       </c>
       <c r="F42" s="10" t="n">
-        <v>1872000</v>
+        <v>1838160</v>
       </c>
       <c r="G42" s="10" t="n">
-        <v>1872000</v>
+        <v>1838160</v>
       </c>
       <c r="H42" s="11">
         <f>F42-G42</f>
@@ -2475,7 +2487,11 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="K42" s="12" t="inlineStr"/>
+      <c r="K42" s="12" t="inlineStr">
+        <is>
+          <t>€36 000</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n">
@@ -2500,7 +2516,7 @@
         </is>
       </c>
       <c r="F43" s="10" t="n">
-        <v>7800000</v>
+        <v>7659000</v>
       </c>
       <c r="G43" s="10" t="n">
         <v>0</v>
@@ -2519,7 +2535,11 @@
           <t>2026-06</t>
         </is>
       </c>
-      <c r="K43" s="12" t="inlineStr"/>
+      <c r="K43" s="12" t="inlineStr">
+        <is>
+          <t>€150 000</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n">
@@ -4104,7 +4124,7 @@
         </is>
       </c>
       <c r="E3" s="11" t="n">
-        <v>7800000</v>
+        <v>7659000</v>
       </c>
       <c r="F3" s="11" t="n">
         <v>0</v>
@@ -4132,7 +4152,7 @@
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>4524000</v>
+        <v>4442220</v>
       </c>
       <c r="F4" s="11" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
4766: 3rd payment received (re-export), overdue cashflow -4.4M
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3119,19 +3119,19 @@
     </row>
     <row r="57">
       <c r="A57" s="8" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="B57" s="9" t="n">
-        <v>3456</v>
+        <v>4766</v>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>А Підселання фундаменту</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E57" s="9" t="inlineStr">
@@ -3140,10 +3140,10 @@
         </is>
       </c>
       <c r="F57" s="10" t="n">
-        <v>335974.68</v>
+        <v>4368478.98</v>
       </c>
       <c r="G57" s="10" t="n">
-        <v>0</v>
+        <v>4368478.98</v>
       </c>
       <c r="H57" s="11">
         <f>F57-G57</f>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="I57" s="9" t="inlineStr">
         <is>
-          <t>прострочено</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3166,11 +3166,11 @@
         <v>46225</v>
       </c>
       <c r="B58" s="9" t="n">
-        <v>5910</v>
+        <v>3456</v>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>А   AGM 2V</t>
+          <t>А Підселання фундаменту</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
@@ -3180,14 +3180,14 @@
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Авансовий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F58" s="10" t="n">
-        <v>8531651.142000001</v>
+        <v>335974.68</v>
       </c>
       <c r="G58" s="10" t="n">
-        <v>8531651.142000001</v>
+        <v>0</v>
       </c>
       <c r="H58" s="11">
         <f>F58-G58</f>
@@ -3195,7 +3195,7 @@
       </c>
       <c r="I58" s="9" t="inlineStr">
         <is>
-          <t>отримано</t>
+          <t>прострочено</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3203,39 +3203,35 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="K58" s="12" t="inlineStr">
-        <is>
-          <t>€167 091</t>
-        </is>
-      </c>
+      <c r="K58" s="12" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n">
-        <v>46227</v>
+        <v>46225</v>
       </c>
       <c r="B59" s="9" t="n">
-        <v>4766</v>
+        <v>5910</v>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>А   AGM 2V</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F59" s="10" t="n">
-        <v>4368478.98</v>
+        <v>8531651.142000001</v>
       </c>
       <c r="G59" s="10" t="n">
-        <v>0</v>
+        <v>8531651.142000001</v>
       </c>
       <c r="H59" s="11">
         <f>F59-G59</f>
@@ -3243,7 +3239,7 @@
       </c>
       <c r="I59" s="9" t="inlineStr">
         <is>
-          <t>прострочено</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3251,7 +3247,11 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="K59" s="12" t="inlineStr"/>
+      <c r="K59" s="12" t="inlineStr">
+        <is>
+          <t>€167 091</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
@@ -4029,7 +4029,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4136,26 +4136,26 @@
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
-        <v>46227</v>
+        <v>46113</v>
       </c>
       <c r="B4" s="9" t="n">
-        <v>4766</v>
+        <v>7068</v>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>А Remtec energy  AGM  160 TP</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="E4" s="11" t="n">
-        <v>4368478.98</v>
+        <v>5640128</v>
       </c>
       <c r="F4" s="11" t="n">
-        <v>0</v>
+        <v>1692038</v>
       </c>
       <c r="G4" s="11">
         <f>E4-F4</f>
@@ -4164,26 +4164,26 @@
     </row>
     <row r="5">
       <c r="A5" s="8" t="n">
-        <v>46113</v>
+        <v>46225</v>
       </c>
       <c r="B5" s="9" t="n">
-        <v>7068</v>
+        <v>3456</v>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>А Remtec energy  AGM  160 TP</t>
+          <t>А Підселання фундаменту</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Авансовий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>5640128</v>
+        <v>335974.68</v>
       </c>
       <c r="F5" s="11" t="n">
-        <v>1692038</v>
+        <v>0</v>
       </c>
       <c r="G5" s="11">
         <f>E5-F5</f>
@@ -4192,23 +4192,23 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
-        <v>46225</v>
+        <v>46212</v>
       </c>
       <c r="B6" s="9" t="n">
-        <v>3456</v>
+        <v>6406</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>А Підселання фундаменту</t>
+          <t>Максим Яловий Чинадієво</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>335974.68</v>
+        <v>218602</v>
       </c>
       <c r="F6" s="11" t="n">
         <v>0</v>
@@ -4220,14 +4220,14 @@
     </row>
     <row r="7">
       <c r="A7" s="8" t="n">
-        <v>46212</v>
+        <v>46213</v>
       </c>
       <c r="B7" s="9" t="n">
-        <v>6406</v>
+        <v>8188</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Максим Яловий Чинадієво</t>
+          <t>Фундамент Ужгород Стефанія</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
@@ -4236,7 +4236,7 @@
         </is>
       </c>
       <c r="E7" s="11" t="n">
-        <v>218602</v>
+        <v>73926</v>
       </c>
       <c r="F7" s="11" t="n">
         <v>0</v>
@@ -4247,54 +4247,26 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="n">
-        <v>46213</v>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>8188</v>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Фундамент Ужгород Стефанія</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Другий платіж</t>
-        </is>
-      </c>
-      <c r="E8" s="11" t="n">
-        <v>73926</v>
-      </c>
-      <c r="F8" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="11">
-        <f>E8-F8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9">
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="E9" s="13">
-        <f>SUM(E2:E8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="13">
-        <f>SUM(F2:F8)</f>
-        <v/>
-      </c>
-      <c r="G9" s="13">
-        <f>SUM(G2:G8)</f>
+      <c r="E8" s="13">
+        <f>SUM(E2:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="13">
+        <f>SUM(F2:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="13">
+        <f>SUM(G2:G7)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G8"/>
+  <autoFilter ref="A1:G7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add 2 new Donska projects 6352 & 8898 (from passports)
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прострочені" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$71</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Дані: 27.07.2026 · без проєктів на паузі/втрачених</t>
+          <t>Дані: 28.07.2026 · без проєктів на паузі/втрачених</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K72"/>
+  <dimension ref="A1:K81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2811,31 +2811,31 @@
     </row>
     <row r="50">
       <c r="A50" s="8" t="n">
-        <v>46217</v>
+        <v>46216</v>
       </c>
       <c r="B50" s="9" t="n">
-        <v>4766</v>
+        <v>8898</v>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>(6022-26 - ГШ Фундамент домобудування)</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F50" s="10" t="n">
-        <v>100000</v>
+        <v>259395.65</v>
       </c>
       <c r="G50" s="10" t="n">
-        <v>100000</v>
+        <v>259395.65</v>
       </c>
       <c r="H50" s="11">
         <f>F50-G50</f>
@@ -2858,16 +2858,16 @@
         <v>46217</v>
       </c>
       <c r="B51" s="9" t="n">
-        <v>8185</v>
+        <v>4766</v>
       </c>
       <c r="C51" s="9" t="inlineStr">
         <is>
-          <t>Фундамент Hytte House Development Славське</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D51" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr">
@@ -2876,10 +2876,10 @@
         </is>
       </c>
       <c r="F51" s="10" t="n">
-        <v>63313.4</v>
+        <v>100000</v>
       </c>
       <c r="G51" s="10" t="n">
-        <v>63313.4</v>
+        <v>100000</v>
       </c>
       <c r="H51" s="11">
         <f>F51-G51</f>
@@ -2916,7 +2916,7 @@
       </c>
       <c r="E52" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F52" s="10" t="n">
@@ -2943,14 +2943,14 @@
     </row>
     <row r="53">
       <c r="A53" s="8" t="n">
-        <v>46219</v>
+        <v>46217</v>
       </c>
       <c r="B53" s="9" t="n">
-        <v>7002</v>
+        <v>8185</v>
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP W 24PS V1</t>
+          <t>Фундамент Hytte House Development Славське</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
@@ -2960,14 +2960,14 @@
       </c>
       <c r="E53" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F53" s="10" t="n">
-        <v>126896.64</v>
+        <v>63313.4</v>
       </c>
       <c r="G53" s="10" t="n">
-        <v>126896.64</v>
+        <v>63313.4</v>
       </c>
       <c r="H53" s="11">
         <f>F53-G53</f>
@@ -2990,11 +2990,11 @@
         <v>46219</v>
       </c>
       <c r="B54" s="9" t="n">
-        <v>7002</v>
+        <v>6352</v>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP W 24PS V1</t>
+          <t>А АБМК ТОВ  SCP Blade 10PS</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
@@ -3004,14 +3004,14 @@
       </c>
       <c r="E54" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F54" s="10" t="n">
-        <v>126896.64</v>
+        <v>80000.03999999999</v>
       </c>
       <c r="G54" s="10" t="n">
-        <v>126896.64</v>
+        <v>80000.03999999999</v>
       </c>
       <c r="H54" s="11">
         <f>F54-G54</f>
@@ -3048,14 +3048,14 @@
       </c>
       <c r="E55" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F55" s="10" t="n">
-        <v>573945</v>
+        <v>126896.64</v>
       </c>
       <c r="G55" s="10" t="n">
-        <v>573945</v>
+        <v>126896.64</v>
       </c>
       <c r="H55" s="11">
         <f>F55-G55</f>
@@ -3075,19 +3075,19 @@
     </row>
     <row r="56">
       <c r="A56" s="8" t="n">
-        <v>46224</v>
+        <v>46219</v>
       </c>
       <c r="B56" s="9" t="n">
-        <v>4766</v>
+        <v>7002</v>
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>А Фора  SCP W 24PS V1</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E56" s="9" t="inlineStr">
@@ -3096,10 +3096,10 @@
         </is>
       </c>
       <c r="F56" s="10" t="n">
-        <v>4368478.98</v>
+        <v>126896.64</v>
       </c>
       <c r="G56" s="10" t="n">
-        <v>4368478.98</v>
+        <v>126896.64</v>
       </c>
       <c r="H56" s="11">
         <f>F56-G56</f>
@@ -3119,14 +3119,14 @@
     </row>
     <row r="57">
       <c r="A57" s="8" t="n">
-        <v>46225</v>
+        <v>46219</v>
       </c>
       <c r="B57" s="9" t="n">
-        <v>3456</v>
+        <v>7002</v>
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>А Підселання фундаменту</t>
+          <t>А Фора  SCP W 24PS V1</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
@@ -3136,14 +3136,14 @@
       </c>
       <c r="E57" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F57" s="10" t="n">
-        <v>335974.68</v>
+        <v>573945</v>
       </c>
       <c r="G57" s="10" t="n">
-        <v>0</v>
+        <v>573945</v>
       </c>
       <c r="H57" s="11">
         <f>F57-G57</f>
@@ -3151,7 +3151,7 @@
       </c>
       <c r="I57" s="9" t="inlineStr">
         <is>
-          <t>прострочено</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3163,31 +3163,31 @@
     </row>
     <row r="58">
       <c r="A58" s="8" t="n">
-        <v>46225</v>
+        <v>46224</v>
       </c>
       <c r="B58" s="9" t="n">
-        <v>5910</v>
+        <v>4766</v>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>А   AGM 2V</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E58" s="9" t="inlineStr">
         <is>
-          <t>Авансовий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F58" s="10" t="n">
-        <v>8516612.979</v>
+        <v>4368478.98</v>
       </c>
       <c r="G58" s="10" t="n">
-        <v>8516612.979</v>
+        <v>4368478.98</v>
       </c>
       <c r="H58" s="11">
         <f>F58-G58</f>
@@ -3203,22 +3203,18 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="K58" s="12" t="inlineStr">
-        <is>
-          <t>€167 091</t>
-        </is>
-      </c>
+      <c r="K58" s="12" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n">
-        <v>46231</v>
+        <v>46225</v>
       </c>
       <c r="B59" s="9" t="n">
-        <v>7894</v>
+        <v>3456</v>
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>А Підселання фундаменту</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
@@ -3228,11 +3224,11 @@
       </c>
       <c r="E59" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F59" s="10" t="n">
-        <v>737597.4</v>
+        <v>335974.68</v>
       </c>
       <c r="G59" s="10" t="n">
         <v>0</v>
@@ -3243,7 +3239,7 @@
       </c>
       <c r="I59" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>прострочено</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3255,31 +3251,31 @@
     </row>
     <row r="60">
       <c r="A60" s="8" t="n">
-        <v>46234</v>
+        <v>46225</v>
       </c>
       <c r="B60" s="9" t="n">
-        <v>7068</v>
+        <v>5910</v>
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>А Remtec energy  AGM  160 TP</t>
+          <t>А   AGM 2V</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
         <is>
-          <t>Александров</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E60" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F60" s="10" t="n">
-        <v>0</v>
+        <v>8516612.979</v>
       </c>
       <c r="G60" s="10" t="n">
-        <v>2794670</v>
+        <v>8516612.979</v>
       </c>
       <c r="H60" s="11">
         <f>F60-G60</f>
@@ -3287,7 +3283,7 @@
       </c>
       <c r="I60" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -3295,32 +3291,36 @@
           <t>2026-07</t>
         </is>
       </c>
-      <c r="K60" s="12" t="inlineStr"/>
+      <c r="K60" s="12" t="inlineStr">
+        <is>
+          <t>€167 091</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n">
-        <v>46234</v>
+        <v>46231</v>
       </c>
       <c r="B61" s="9" t="n">
-        <v>7244</v>
+        <v>7894</v>
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>В Модулекс модульна будівля Чернігів</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E61" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F61" s="10" t="n">
-        <v>132708.6</v>
+        <v>737597.4</v>
       </c>
       <c r="G61" s="10" t="n">
         <v>0</v>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="I61" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>прострочено</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
@@ -3343,19 +3343,19 @@
     </row>
     <row r="62">
       <c r="A62" s="8" t="n">
-        <v>46237</v>
+        <v>46232</v>
       </c>
       <c r="B62" s="9" t="n">
-        <v>6406</v>
+        <v>8898</v>
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Максим Яловий Чинадієво</t>
+          <t>(6022-26 - ГШ Фундамент домобудування)</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
         <is>
-          <t>Іщук</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E62" s="9" t="inlineStr">
@@ -3364,7 +3364,7 @@
         </is>
       </c>
       <c r="F62" s="10" t="n">
-        <v>218602</v>
+        <v>27768</v>
       </c>
       <c r="G62" s="10" t="n">
         <v>0</v>
@@ -3380,38 +3380,38 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="K62" s="12" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n">
-        <v>46237</v>
+        <v>46234</v>
       </c>
       <c r="B63" s="9" t="n">
-        <v>7894</v>
+        <v>7068</v>
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>А Remtec energy  AGM  160 TP</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Александров</t>
         </is>
       </c>
       <c r="E63" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F63" s="10" t="n">
-        <v>185968</v>
+        <v>0</v>
       </c>
       <c r="G63" s="10" t="n">
-        <v>0</v>
+        <v>2794670</v>
       </c>
       <c r="H63" s="11">
         <f>F63-G63</f>
@@ -3424,21 +3424,21 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="K63" s="12" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="8" t="n">
-        <v>46237</v>
+        <v>46234</v>
       </c>
       <c r="B64" s="9" t="n">
-        <v>8878</v>
+        <v>7244</v>
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
+          <t>В Модулекс модульна будівля Чернігів</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -3452,7 +3452,7 @@
         </is>
       </c>
       <c r="F64" s="10" t="n">
-        <v>12823</v>
+        <v>132708.6</v>
       </c>
       <c r="G64" s="10" t="n">
         <v>0</v>
@@ -3468,21 +3468,21 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="K64" s="12" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="8" t="n">
-        <v>46245</v>
+        <v>46237</v>
       </c>
       <c r="B65" s="9" t="n">
-        <v>7894</v>
+        <v>6352</v>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>А АБМК ТОВ  SCP Blade 10PS</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -3492,11 +3492,11 @@
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F65" s="10" t="n">
-        <v>185967.99</v>
+        <v>1399046.58</v>
       </c>
       <c r="G65" s="10" t="n">
         <v>0</v>
@@ -3519,19 +3519,19 @@
     </row>
     <row r="66">
       <c r="A66" s="8" t="n">
-        <v>46247</v>
+        <v>46237</v>
       </c>
       <c r="B66" s="9" t="n">
-        <v>5910</v>
+        <v>6406</v>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>А   AGM 2V</t>
+          <t>Максим Яловий Чинадієво</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Іщук</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
@@ -3540,7 +3540,7 @@
         </is>
       </c>
       <c r="F66" s="10" t="n">
-        <v>17033225.958</v>
+        <v>218602</v>
       </c>
       <c r="G66" s="10" t="n">
         <v>0</v>
@@ -3559,22 +3559,18 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K66" s="12" t="inlineStr">
-        <is>
-          <t>€334 181</t>
-        </is>
-      </c>
+      <c r="K66" s="12" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="8" t="n">
-        <v>46260</v>
+        <v>46237</v>
       </c>
       <c r="B67" s="9" t="n">
-        <v>7002</v>
+        <v>7894</v>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP W 24PS V1</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
@@ -3584,11 +3580,11 @@
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F67" s="10" t="n">
-        <v>573945</v>
+        <v>185968</v>
       </c>
       <c r="G67" s="10" t="n">
         <v>0</v>
@@ -3611,14 +3607,14 @@
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
-        <v>46266</v>
+        <v>46237</v>
       </c>
       <c r="B68" s="9" t="n">
-        <v>4766</v>
+        <v>8878</v>
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -3628,11 +3624,11 @@
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F68" s="10" t="n">
-        <v>128100</v>
+        <v>12823</v>
       </c>
       <c r="G68" s="10" t="n">
         <v>0</v>
@@ -3648,35 +3644,35 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="K68" s="12" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
-        <v>46267</v>
+        <v>46245</v>
       </c>
       <c r="B69" s="9" t="n">
-        <v>4766</v>
+        <v>7894</v>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F69" s="10" t="n">
-        <v>1199397.42</v>
+        <v>185967.99</v>
       </c>
       <c r="G69" s="10" t="n">
         <v>0</v>
@@ -3692,14 +3688,14 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="K69" s="12" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
-        <v>46279</v>
+        <v>46247</v>
       </c>
       <c r="B70" s="9" t="n">
         <v>5910</v>
@@ -3716,11 +3712,11 @@
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F70" s="10" t="n">
-        <v>2838870.993</v>
+        <v>17033225.958</v>
       </c>
       <c r="G70" s="10" t="n">
         <v>0</v>
@@ -3736,25 +3732,25 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="K70" s="12" t="inlineStr">
         <is>
-          <t>€55 697</t>
+          <t>€334 181</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n">
-        <v>46282</v>
+        <v>46248</v>
       </c>
       <c r="B71" s="9" t="n">
-        <v>7894</v>
+        <v>8898</v>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>(6022-26 - ГШ Фундамент домобудування)</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
@@ -3764,11 +3760,11 @@
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F71" s="10" t="n">
-        <v>737597.4</v>
+        <v>189603.75</v>
       </c>
       <c r="G71" s="10" t="n">
         <v>0</v>
@@ -3784,32 +3780,428 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="K71" s="12" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="8" t="n">
+        <v>46260</v>
+      </c>
+      <c r="B72" s="9" t="n">
+        <v>7002</v>
+      </c>
+      <c r="C72" s="9" t="inlineStr">
+        <is>
+          <t>А Фора  SCP W 24PS V1</t>
+        </is>
+      </c>
+      <c r="D72" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E72" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F72" s="10" t="n">
+        <v>573945</v>
+      </c>
+      <c r="G72" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" s="11">
+        <f>F72-G72</f>
+        <v/>
+      </c>
+      <c r="I72" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="K72" s="12" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="8" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B73" s="9" t="n">
+        <v>4766</v>
+      </c>
+      <c r="C73" s="9" t="inlineStr">
+        <is>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
+        </is>
+      </c>
+      <c r="D73" s="9" t="inlineStr">
+        <is>
+          <t>Заянчковський</t>
+        </is>
+      </c>
+      <c r="E73" s="9" t="inlineStr">
+        <is>
+          <t>Четвертий платіж</t>
+        </is>
+      </c>
+      <c r="F73" s="10" t="n">
+        <v>128100</v>
+      </c>
+      <c r="G73" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" s="11">
+        <f>F73-G73</f>
+        <v/>
+      </c>
+      <c r="I73" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
           <t>2026-09</t>
         </is>
       </c>
-      <c r="K71" s="12" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="E72" s="3" t="inlineStr">
+      <c r="K73" s="12" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="8" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B74" s="9" t="n">
+        <v>8898</v>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>(6022-26 - ГШ Фундамент домобудування)</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E74" s="9" t="inlineStr">
+        <is>
+          <t>Четвертий платіж</t>
+        </is>
+      </c>
+      <c r="F74" s="10" t="n">
+        <v>189603.75</v>
+      </c>
+      <c r="G74" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" s="11">
+        <f>F74-G74</f>
+        <v/>
+      </c>
+      <c r="I74" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K74" s="12" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="8" t="n">
+        <v>46267</v>
+      </c>
+      <c r="B75" s="9" t="n">
+        <v>4766</v>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>Заянчковський</t>
+        </is>
+      </c>
+      <c r="E75" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F75" s="10" t="n">
+        <v>1199397.42</v>
+      </c>
+      <c r="G75" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" s="11">
+        <f>F75-G75</f>
+        <v/>
+      </c>
+      <c r="I75" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K75" s="12" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B76" s="9" t="n">
+        <v>5910</v>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>А   AGM 2V</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E76" s="9" t="inlineStr">
+        <is>
+          <t>Третій платіж</t>
+        </is>
+      </c>
+      <c r="F76" s="10" t="n">
+        <v>2838870.993</v>
+      </c>
+      <c r="G76" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" s="11">
+        <f>F76-G76</f>
+        <v/>
+      </c>
+      <c r="I76" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K76" s="12" t="inlineStr">
+        <is>
+          <t>€55 697</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="8" t="n">
+        <v>46282</v>
+      </c>
+      <c r="B77" s="9" t="n">
+        <v>7894</v>
+      </c>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>А Фора  SCP  32PS</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E77" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F77" s="10" t="n">
+        <v>737597.4</v>
+      </c>
+      <c r="G77" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" s="11">
+        <f>F77-G77</f>
+        <v/>
+      </c>
+      <c r="I77" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K77" s="12" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="8" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B78" s="9" t="n">
+        <v>6352</v>
+      </c>
+      <c r="C78" s="9" t="inlineStr">
+        <is>
+          <t>А АБМК ТОВ  SCP Blade 10PS</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E78" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F78" s="10" t="n">
+        <v>651792.28</v>
+      </c>
+      <c r="G78" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" s="11">
+        <f>F78-G78</f>
+        <v/>
+      </c>
+      <c r="I78" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="K78" s="12" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="8" t="n"/>
+      <c r="B79" s="9" t="n">
+        <v>6352</v>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>А АБМК ТОВ  SCP Blade 10PS</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E79" s="9" t="inlineStr">
+        <is>
+          <t>Третій платіж</t>
+        </is>
+      </c>
+      <c r="F79" s="10" t="n">
+        <v>1119237.26</v>
+      </c>
+      <c r="G79" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" s="11">
+        <f>F79-G79</f>
+        <v/>
+      </c>
+      <c r="I79" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>без дати</t>
+        </is>
+      </c>
+      <c r="K79" s="12" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="8" t="n"/>
+      <c r="B80" s="9" t="n">
+        <v>6352</v>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>А АБМК ТОВ  SCP Blade 10PS</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E80" s="9" t="inlineStr">
+        <is>
+          <t>Четвертий платіж</t>
+        </is>
+      </c>
+      <c r="F80" s="10" t="n">
+        <v>371982.96</v>
+      </c>
+      <c r="G80" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" s="11">
+        <f>F80-G80</f>
+        <v/>
+      </c>
+      <c r="I80" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>без дати</t>
+        </is>
+      </c>
+      <c r="K80" s="12" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="E81" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="F72" s="13">
-        <f>SUM(F2:F71)</f>
-        <v/>
-      </c>
-      <c r="G72" s="13">
-        <f>SUM(G2:G71)</f>
-        <v/>
-      </c>
-      <c r="H72" s="13">
-        <f>SUM(H2:H71)</f>
+      <c r="F81" s="13">
+        <f>SUM(F2:F80)</f>
+        <v/>
+      </c>
+      <c r="G81" s="13">
+        <f>SUM(G2:G80)</f>
+        <v/>
+      </c>
+      <c r="H81" s="13">
+        <f>SUM(H2:H80)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I71"/>
+  <autoFilter ref="A1:I80"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3820,7 +4212,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3996,25 +4388,71 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>жов 2026</t>
+        </is>
+      </c>
+      <c r="B8" s="11">
+        <f>SUMIF('Графік надходжень'!J:J,"2026-10",'Графік надходжень'!F:F)</f>
+        <v/>
+      </c>
+      <c r="C8" s="11">
+        <f>SUMIF('Графік надходжень'!J:J,"2026-10",'Графік надходжень'!G:G)</f>
+        <v/>
+      </c>
+      <c r="D8" s="11">
+        <f>B8-C8</f>
+        <v/>
+      </c>
+      <c r="E8" s="14">
+        <f>IF(B8=0,0,C8/B8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>без дати</t>
+        </is>
+      </c>
+      <c r="B9" s="11">
+        <f>SUMIF('Графік надходжень'!J:J,"без дати",'Графік надходжень'!F:F)</f>
+        <v/>
+      </c>
+      <c r="C9" s="11">
+        <f>SUMIF('Графік надходжень'!J:J,"без дати",'Графік надходжень'!G:G)</f>
+        <v/>
+      </c>
+      <c r="D9" s="11">
+        <f>B9-C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="14">
+        <f>IF(B9=0,0,C9/B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="B8" s="13">
-        <f>SUM(B2:B7)</f>
-        <v/>
-      </c>
-      <c r="C8" s="13">
-        <f>SUM(C2:C7)</f>
-        <v/>
-      </c>
-      <c r="D8" s="13">
-        <f>SUM(D2:D7)</f>
-        <v/>
-      </c>
-      <c r="E8" s="15">
-        <f>IF(B8=0,0,C8/B8)</f>
+      <c r="B10" s="13">
+        <f>SUM(B2:B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="13">
+        <f>SUM(C2:C9)</f>
+        <v/>
+      </c>
+      <c r="D10" s="13">
+        <f>SUM(D2:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="15">
+        <f>IF(B10=0,0,C10/B10)</f>
         <v/>
       </c>
     </row>
@@ -4029,7 +4467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4164,23 +4602,23 @@
     </row>
     <row r="5">
       <c r="A5" s="8" t="n">
-        <v>46225</v>
+        <v>46231</v>
       </c>
       <c r="B5" s="9" t="n">
-        <v>3456</v>
+        <v>7894</v>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>А Підселання фундаменту</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="E5" s="11" t="n">
-        <v>335974.68</v>
+        <v>737597.4</v>
       </c>
       <c r="F5" s="11" t="n">
         <v>0</v>
@@ -4192,23 +4630,23 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="n">
-        <v>46213</v>
+        <v>46225</v>
       </c>
       <c r="B6" s="9" t="n">
-        <v>8188</v>
+        <v>3456</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Фундамент Ужгород Стефанія</t>
+          <t>А Підселання фундаменту</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="E6" s="11" t="n">
-        <v>73926</v>
+        <v>335974.68</v>
       </c>
       <c r="F6" s="11" t="n">
         <v>0</v>
@@ -4219,26 +4657,54 @@
       </c>
     </row>
     <row r="7">
-      <c r="D7" s="3" t="inlineStr">
+      <c r="A7" s="8" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>8188</v>
+      </c>
+      <c r="C7" s="9" t="inlineStr">
+        <is>
+          <t>Фундамент Ужгород Стефанія</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
+          <t>Другий платіж</t>
+        </is>
+      </c>
+      <c r="E7" s="11" t="n">
+        <v>73926</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="11">
+        <f>E7-F7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="E7" s="13">
-        <f>SUM(E2:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="13">
-        <f>SUM(F2:F6)</f>
-        <v/>
-      </c>
-      <c r="G7" s="13">
-        <f>SUM(G2:G6)</f>
+      <c r="E8" s="13">
+        <f>SUM(E2:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="13">
+        <f>SUM(F2:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="13">
+        <f>SUM(G2:G7)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G6"/>
+  <autoFilter ref="A1:G7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
6352 & 8898: real Planner exports (budgets, full tasks, pct 0%)
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -2818,7 +2818,7 @@
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>(6022-26 - ГШ Фундамент домобудування)</t>
+          <t>6022-26 - ГШ Фундамент домобудування</t>
         </is>
       </c>
       <c r="D50" s="9" t="inlineStr">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>(6022-26 - ГШ Фундамент домобудування)</t>
+          <t>6022-26 - ГШ Фундамент домобудування</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
@@ -3743,14 +3743,14 @@
     </row>
     <row r="71">
       <c r="A71" s="8" t="n">
-        <v>46248</v>
+        <v>46258</v>
       </c>
       <c r="B71" s="9" t="n">
-        <v>8898</v>
+        <v>6352</v>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>(6022-26 - ГШ Фундамент домобудування)</t>
+          <t>А АБМК ТОВ  SCP Blade 10PS</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
@@ -3764,7 +3764,7 @@
         </is>
       </c>
       <c r="F71" s="10" t="n">
-        <v>189603.75</v>
+        <v>1119237.26</v>
       </c>
       <c r="G71" s="10" t="n">
         <v>0</v>
@@ -3875,28 +3875,28 @@
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
-        <v>46266</v>
+        <v>46267</v>
       </c>
       <c r="B74" s="9" t="n">
-        <v>8898</v>
+        <v>4766</v>
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>(6022-26 - ГШ Фундамент домобудування)</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F74" s="10" t="n">
-        <v>189603.75</v>
+        <v>1199397.42</v>
       </c>
       <c r="G74" s="10" t="n">
         <v>0</v>
@@ -3922,25 +3922,25 @@
         <v>46267</v>
       </c>
       <c r="B75" s="9" t="n">
-        <v>4766</v>
+        <v>8898</v>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>6022-26 - ГШ Фундамент домобудування</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F75" s="10" t="n">
-        <v>1199397.42</v>
+        <v>189603.75</v>
       </c>
       <c r="G75" s="10" t="n">
         <v>0</v>
@@ -4011,14 +4011,14 @@
     </row>
     <row r="77">
       <c r="A77" s="8" t="n">
-        <v>46282</v>
+        <v>46280</v>
       </c>
       <c r="B77" s="9" t="n">
-        <v>7894</v>
+        <v>8898</v>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>А Фора  SCP  32PS</t>
+          <t>6022-26 - ГШ Фундамент домобудування</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
@@ -4028,11 +4028,11 @@
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F77" s="10" t="n">
-        <v>737597.4</v>
+        <v>189603.75</v>
       </c>
       <c r="G77" s="10" t="n">
         <v>0</v>
@@ -4055,14 +4055,14 @@
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>46320</v>
+        <v>46282</v>
       </c>
       <c r="B78" s="9" t="n">
-        <v>6352</v>
+        <v>7894</v>
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>А АБМК ТОВ  SCP Blade 10PS</t>
+          <t>А Фора  SCP  32PS</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
@@ -4076,7 +4076,7 @@
         </is>
       </c>
       <c r="F78" s="10" t="n">
-        <v>651792.28</v>
+        <v>737597.4</v>
       </c>
       <c r="G78" s="10" t="n">
         <v>0</v>
@@ -4092,13 +4092,15 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="K78" s="12" t="inlineStr"/>
     </row>
     <row r="79">
-      <c r="A79" s="8" t="n"/>
+      <c r="A79" s="8" t="n">
+        <v>46308</v>
+      </c>
       <c r="B79" s="9" t="n">
         <v>6352</v>
       </c>
@@ -4114,11 +4116,11 @@
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>1119237.26</v>
+        <v>371982.96</v>
       </c>
       <c r="G79" s="10" t="n">
         <v>0</v>
@@ -4134,13 +4136,15 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>без дати</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="K79" s="12" t="inlineStr"/>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="n"/>
+      <c r="A80" s="8" t="n">
+        <v>46321</v>
+      </c>
       <c r="B80" s="9" t="n">
         <v>6352</v>
       </c>
@@ -4156,11 +4160,11 @@
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F80" s="10" t="n">
-        <v>371982.96</v>
+        <v>651792.28</v>
       </c>
       <c r="G80" s="10" t="n">
         <v>0</v>
@@ -4176,7 +4180,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>без дати</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="K80" s="12" t="inlineStr"/>
@@ -4212,7 +4216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4411,48 +4415,25 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>без дати</t>
-        </is>
-      </c>
-      <c r="B9" s="11">
-        <f>SUMIF('Графік надходжень'!J:J,"без дати",'Графік надходжень'!F:F)</f>
-        <v/>
-      </c>
-      <c r="C9" s="11">
-        <f>SUMIF('Графік надходжень'!J:J,"без дати",'Графік надходжень'!G:G)</f>
-        <v/>
-      </c>
-      <c r="D9" s="11">
-        <f>B9-C9</f>
-        <v/>
-      </c>
-      <c r="E9" s="14">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Разом</t>
+        </is>
+      </c>
+      <c r="B9" s="13">
+        <f>SUM(B2:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="13">
+        <f>SUM(C2:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="13">
+        <f>SUM(D2:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="15">
         <f>IF(B9=0,0,C9/B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Разом</t>
-        </is>
-      </c>
-      <c r="B10" s="13">
-        <f>SUM(B2:B9)</f>
-        <v/>
-      </c>
-      <c r="C10" s="13">
-        <f>SUM(C2:C9)</f>
-        <v/>
-      </c>
-      <c r="D10" s="13">
-        <f>SUM(D2:D9)</f>
-        <v/>
-      </c>
-      <c r="E10" s="15">
-        <f>IF(B10=0,0,C10/B10)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
5870 budget update 18.08.2026 (Третій 14575 paid, Четвертий 17500 debt) + portfolio/PM/cashflow
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прострочені" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K84"/>
+  <dimension ref="A1:K85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3475,31 +3475,31 @@
     </row>
     <row r="65">
       <c r="A65" s="8" t="n">
-        <v>46253</v>
+        <v>46241</v>
       </c>
       <c r="B65" s="9" t="n">
-        <v>8898</v>
+        <v>5870</v>
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>Григорівка №3</t>
+          <t>Carport Airport Munich</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E65" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F65" s="10" t="n">
-        <v>188043.75</v>
+        <v>753673.25</v>
       </c>
       <c r="G65" s="10" t="n">
-        <v>0</v>
+        <v>753673.25</v>
       </c>
       <c r="H65" s="11">
         <f>F65-G65</f>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="I65" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3515,32 +3515,36 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K65" s="12" t="inlineStr"/>
+      <c r="K65" s="12" t="inlineStr">
+        <is>
+          <t>€14 575</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="n">
-        <v>46255</v>
+        <v>46253</v>
       </c>
       <c r="B66" s="9" t="n">
-        <v>8878</v>
+        <v>8898</v>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
+          <t>Григорівка №3</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E66" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F66" s="10" t="n">
-        <v>12823</v>
+        <v>188043.75</v>
       </c>
       <c r="G66" s="10" t="n">
         <v>0</v>
@@ -3563,28 +3567,28 @@
     </row>
     <row r="67">
       <c r="A67" s="8" t="n">
-        <v>46258</v>
+        <v>46255</v>
       </c>
       <c r="B67" s="9" t="n">
-        <v>3456</v>
+        <v>8878</v>
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>А Підселання фундаменту</t>
+          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E67" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F67" s="10" t="n">
-        <v>335974.68</v>
+        <v>12823</v>
       </c>
       <c r="G67" s="10" t="n">
         <v>0</v>
@@ -3610,11 +3614,11 @@
         <v>46258</v>
       </c>
       <c r="B68" s="9" t="n">
-        <v>6352</v>
+        <v>3456</v>
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>АБМК SCP Blade 8PS</t>
+          <t>А Підселання фундаменту</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -3628,7 +3632,7 @@
         </is>
       </c>
       <c r="F68" s="10" t="n">
-        <v>1119237.26</v>
+        <v>335974.68</v>
       </c>
       <c r="G68" s="10" t="n">
         <v>0</v>
@@ -3651,28 +3655,28 @@
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
-        <v>46259</v>
+        <v>46258</v>
       </c>
       <c r="B69" s="9" t="n">
-        <v>6406</v>
+        <v>6352</v>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>Максим Яловий Чинадієво</t>
+          <t>АБМК SCP Blade 8PS</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Іщук</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F69" s="10" t="n">
-        <v>218602</v>
+        <v>1119237.26</v>
       </c>
       <c r="G69" s="10" t="n">
         <v>0</v>
@@ -3695,31 +3699,31 @@
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
-        <v>46261</v>
+        <v>46259</v>
       </c>
       <c r="B70" s="9" t="n">
-        <v>5910</v>
+        <v>6406</v>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>SGM Brdovec, Хорватия</t>
+          <t>Максим Яловий Чинадієво</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Іщук</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж 60%</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F70" s="10" t="n">
-        <v>17280499.51</v>
+        <v>218602</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>2969188.2</v>
+        <v>0</v>
       </c>
       <c r="H70" s="11">
         <f>F70-G70</f>
@@ -3735,22 +3739,18 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K70" s="12" t="inlineStr">
-        <is>
-          <t>€334 181</t>
-        </is>
-      </c>
+      <c r="K70" s="12" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="8" t="n">
-        <v>46262</v>
+        <v>46261</v>
       </c>
       <c r="B71" s="9" t="n">
-        <v>7894</v>
+        <v>5910</v>
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>SCP Фора  Хотів</t>
+          <t>SGM Brdovec, Хорватия</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
@@ -3760,14 +3760,14 @@
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Другий платіж 60%</t>
         </is>
       </c>
       <c r="F71" s="10" t="n">
-        <v>185968</v>
+        <v>17280499.51</v>
       </c>
       <c r="G71" s="10" t="n">
-        <v>0</v>
+        <v>2969188.2</v>
       </c>
       <c r="H71" s="11">
         <f>F71-G71</f>
@@ -3783,32 +3783,36 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K71" s="12" t="inlineStr"/>
+      <c r="K71" s="12" t="inlineStr">
+        <is>
+          <t>€334 181</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="8" t="n">
-        <v>46263</v>
+        <v>46262</v>
       </c>
       <c r="B72" s="9" t="n">
-        <v>5870</v>
+        <v>7894</v>
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>Carport Airport Munich</t>
+          <t>SCP Фора  Хотів</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Хома</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F72" s="10" t="n">
-        <v>1658598.25</v>
+        <v>185968</v>
       </c>
       <c r="G72" s="10" t="n">
         <v>0</v>
@@ -3827,11 +3831,7 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K72" s="12" t="inlineStr">
-        <is>
-          <t>€32 075</t>
-        </is>
-      </c>
+      <c r="K72" s="12" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="8" t="n">
@@ -3879,31 +3879,31 @@
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
-        <v>46265</v>
+        <v>46264</v>
       </c>
       <c r="B74" s="9" t="n">
-        <v>6130</v>
+        <v>5870</v>
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ Фундамент домобудування Євро Простір Марія</t>
+          <t>Carport Airport Munich</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F74" s="10" t="n">
-        <v>73335</v>
+        <v>904925</v>
       </c>
       <c r="G74" s="10" t="n">
-        <v>36665</v>
+        <v>0</v>
       </c>
       <c r="H74" s="11">
         <f>F74-G74</f>
@@ -3919,18 +3919,22 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K74" s="12" t="inlineStr"/>
+      <c r="K74" s="12" t="inlineStr">
+        <is>
+          <t>€17 500</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
         <v>46265</v>
       </c>
       <c r="B75" s="9" t="n">
-        <v>7244</v>
+        <v>6130</v>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>В Модулекс модульна будівля Чернігів</t>
+          <t>-26 ГШ Фундамент домобудування Євро Простір Марія</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
@@ -3944,10 +3948,10 @@
         </is>
       </c>
       <c r="F75" s="10" t="n">
-        <v>132708.6</v>
+        <v>73335</v>
       </c>
       <c r="G75" s="10" t="n">
-        <v>0</v>
+        <v>36665</v>
       </c>
       <c r="H75" s="11">
         <f>F75-G75</f>
@@ -3967,14 +3971,14 @@
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
-        <v>46267</v>
+        <v>46265</v>
       </c>
       <c r="B76" s="9" t="n">
-        <v>4766</v>
+        <v>7244</v>
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>В Модулекс модульна будівля Чернігів</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
@@ -3988,7 +3992,7 @@
         </is>
       </c>
       <c r="F76" s="10" t="n">
-        <v>1263447.42</v>
+        <v>132708.6</v>
       </c>
       <c r="G76" s="10" t="n">
         <v>0</v>
@@ -4004,7 +4008,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="K76" s="12" t="inlineStr"/>
@@ -4014,25 +4018,25 @@
         <v>46267</v>
       </c>
       <c r="B77" s="9" t="n">
-        <v>5910</v>
+        <v>4766</v>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>SGM Brdovec, Хорватия</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F77" s="10" t="n">
-        <v>2879936.74</v>
+        <v>1263447.42</v>
       </c>
       <c r="G77" s="10" t="n">
         <v>0</v>
@@ -4051,22 +4055,18 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="K77" s="12" t="inlineStr">
-        <is>
-          <t>€55 694</t>
-        </is>
-      </c>
+      <c r="K77" s="12" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>46273</v>
+        <v>46267</v>
       </c>
       <c r="B78" s="9" t="n">
-        <v>7002</v>
+        <v>5910</v>
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>Фора SCP Млиново</t>
+          <t>SGM Brdovec, Хорватия</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
@@ -4076,11 +4076,11 @@
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F78" s="10" t="n">
-        <v>573945</v>
+        <v>2879936.74</v>
       </c>
       <c r="G78" s="10" t="n">
         <v>0</v>
@@ -4099,18 +4099,22 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="K78" s="12" t="inlineStr"/>
+      <c r="K78" s="12" t="inlineStr">
+        <is>
+          <t>€55 694</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n">
-        <v>46280</v>
+        <v>46273</v>
       </c>
       <c r="B79" s="9" t="n">
-        <v>8898</v>
+        <v>7002</v>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>Григорівка №3</t>
+          <t>Фора SCP Млиново</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
@@ -4120,11 +4124,11 @@
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>188043.75</v>
+        <v>573945</v>
       </c>
       <c r="G79" s="10" t="n">
         <v>0</v>
@@ -4147,19 +4151,19 @@
     </row>
     <row r="80">
       <c r="A80" s="8" t="n">
-        <v>46283</v>
+        <v>46280</v>
       </c>
       <c r="B80" s="9" t="n">
-        <v>7508</v>
+        <v>8898</v>
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>8602 Євген Весільна тераса Подорожнє</t>
+          <t>Григорівка №3</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E80" s="9" t="inlineStr">
@@ -4168,7 +4172,7 @@
         </is>
       </c>
       <c r="F80" s="10" t="n">
-        <v>750999.9399999999</v>
+        <v>188043.75</v>
       </c>
       <c r="G80" s="10" t="n">
         <v>0</v>
@@ -4191,28 +4195,28 @@
     </row>
     <row r="81">
       <c r="A81" s="8" t="n">
-        <v>46297</v>
+        <v>46283</v>
       </c>
       <c r="B81" s="9" t="n">
-        <v>7894</v>
+        <v>7508</v>
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>SCP Фора  Хотів</t>
+          <t>8602 Євген Весільна тераса Подорожнє</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F81" s="10" t="n">
-        <v>737597.4</v>
+        <v>750999.9399999999</v>
       </c>
       <c r="G81" s="10" t="n">
         <v>0</v>
@@ -4228,21 +4232,21 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="K81" s="12" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
-        <v>46308</v>
+        <v>46297</v>
       </c>
       <c r="B82" s="9" t="n">
-        <v>6352</v>
+        <v>7894</v>
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>АБМК SCP Blade 8PS</t>
+          <t>SCP Фора  Хотів</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
@@ -4252,11 +4256,11 @@
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F82" s="10" t="n">
-        <v>371982.96</v>
+        <v>737597.4</v>
       </c>
       <c r="G82" s="10" t="n">
         <v>0</v>
@@ -4279,7 +4283,7 @@
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
-        <v>46321</v>
+        <v>46308</v>
       </c>
       <c r="B83" s="9" t="n">
         <v>6352</v>
@@ -4296,11 +4300,11 @@
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F83" s="10" t="n">
-        <v>651792.28</v>
+        <v>371982.96</v>
       </c>
       <c r="G83" s="10" t="n">
         <v>0</v>
@@ -4322,26 +4326,70 @@
       <c r="K83" s="12" t="inlineStr"/>
     </row>
     <row r="84">
-      <c r="E84" s="3" t="inlineStr">
+      <c r="A84" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B84" s="9" t="n">
+        <v>6352</v>
+      </c>
+      <c r="C84" s="9" t="inlineStr">
+        <is>
+          <t>АБМК SCP Blade 8PS</t>
+        </is>
+      </c>
+      <c r="D84" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E84" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F84" s="10" t="n">
+        <v>651792.28</v>
+      </c>
+      <c r="G84" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" s="11">
+        <f>F84-G84</f>
+        <v/>
+      </c>
+      <c r="I84" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="K84" s="12" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="E85" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="F84" s="13">
-        <f>SUM(F2:F83)</f>
-        <v/>
-      </c>
-      <c r="G84" s="13">
-        <f>SUM(G2:G83)</f>
-        <v/>
-      </c>
-      <c r="H84" s="13">
-        <f>SUM(H2:H83)</f>
+      <c r="F85" s="13">
+        <f>SUM(F2:F84)</f>
+        <v/>
+      </c>
+      <c r="G85" s="13">
+        <f>SUM(G2:G84)</f>
+        <v/>
+      </c>
+      <c r="H85" s="13">
+        <f>SUM(H2:H84)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I83"/>
+  <autoFilter ref="A1:I84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Донська update 26.08.2026: 3456 (+20д, план 39%, борг 336к знято), 5910 (61%, overdue 0)
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$90</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3787,28 +3787,28 @@
     </row>
     <row r="72">
       <c r="A72" s="8" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="B72" s="9" t="n">
-        <v>3456</v>
+        <v>6406</v>
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>А Підселання фундаменту</t>
+          <t>Максим Яловий Чинадієво</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Іщук</t>
         </is>
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F72" s="10" t="n">
-        <v>335974.68</v>
+        <v>218602</v>
       </c>
       <c r="G72" s="10" t="n">
         <v>0</v>
@@ -3831,28 +3831,28 @@
     </row>
     <row r="73">
       <c r="A73" s="8" t="n">
-        <v>46259</v>
+        <v>46264</v>
       </c>
       <c r="B73" s="9" t="n">
-        <v>6406</v>
+        <v>5870</v>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>Максим Яловий Чинадієво</t>
+          <t>Carport Airport Munich</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Іщук</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F73" s="10" t="n">
-        <v>218602</v>
+        <v>911575.0000000001</v>
       </c>
       <c r="G73" s="10" t="n">
         <v>0</v>
@@ -3863,7 +3863,7 @@
       </c>
       <c r="I73" s="9" t="inlineStr">
         <is>
-          <t>прострочено</t>
+          <t>очікується</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3871,11 +3871,15 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K73" s="12" t="inlineStr"/>
+      <c r="K73" s="12" t="inlineStr">
+        <is>
+          <t>€17 500</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
-        <v>46263</v>
+        <v>46265</v>
       </c>
       <c r="B74" s="9" t="n">
         <v>5910</v>
@@ -3923,31 +3927,31 @@
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
-        <v>46264</v>
+        <v>46265</v>
       </c>
       <c r="B75" s="9" t="n">
-        <v>5870</v>
+        <v>6130</v>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>Carport Airport Munich</t>
+          <t>-26 ГШ Фундамент домобудування Євро Простір Марія</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Хома</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F75" s="10" t="n">
-        <v>911575.0000000001</v>
+        <v>73335</v>
       </c>
       <c r="G75" s="10" t="n">
-        <v>0</v>
+        <v>36665</v>
       </c>
       <c r="H75" s="11">
         <f>F75-G75</f>
@@ -3963,22 +3967,18 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K75" s="12" t="inlineStr">
-        <is>
-          <t>€17 500</t>
-        </is>
-      </c>
+      <c r="K75" s="12" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
         <v>46265</v>
       </c>
       <c r="B76" s="9" t="n">
-        <v>6130</v>
+        <v>7244</v>
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ Фундамент домобудування Євро Простір Марія</t>
+          <t>В Модулекс модульна будівля Чернігів</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
@@ -3992,10 +3992,10 @@
         </is>
       </c>
       <c r="F76" s="10" t="n">
-        <v>73335</v>
+        <v>132708.6</v>
       </c>
       <c r="G76" s="10" t="n">
-        <v>36665</v>
+        <v>0</v>
       </c>
       <c r="H76" s="11">
         <f>F76-G76</f>
@@ -4018,11 +4018,11 @@
         <v>46265</v>
       </c>
       <c r="B77" s="9" t="n">
-        <v>7244</v>
+        <v>8878</v>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>В Модулекс модульна будівля Чернігів</t>
+          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
@@ -4036,7 +4036,7 @@
         </is>
       </c>
       <c r="F77" s="10" t="n">
-        <v>132708.6</v>
+        <v>12823</v>
       </c>
       <c r="G77" s="10" t="n">
         <v>0</v>
@@ -4059,28 +4059,28 @@
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="B78" s="9" t="n">
-        <v>8878</v>
+        <v>3456</v>
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
+          <t>А Підселання фундаменту</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F78" s="10" t="n">
-        <v>12823</v>
+        <v>335974.68</v>
       </c>
       <c r="G78" s="10" t="n">
         <v>0</v>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="K78" s="12" t="inlineStr"/>
@@ -4896,7 +4896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4947,23 +4947,23 @@
     </row>
     <row r="2">
       <c r="A2" s="8" t="n">
-        <v>46258</v>
+        <v>46259</v>
       </c>
       <c r="B2" s="9" t="n">
-        <v>3456</v>
+        <v>6406</v>
       </c>
       <c r="C2" s="9" t="inlineStr">
         <is>
-          <t>А Підселання фундаменту</t>
+          <t>Максим Яловий Чинадієво</t>
         </is>
       </c>
       <c r="D2" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="E2" s="11" t="n">
-        <v>335974.68</v>
+        <v>218602</v>
       </c>
       <c r="F2" s="11" t="n">
         <v>0</v>
@@ -4974,54 +4974,26 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="n">
-        <v>46259</v>
-      </c>
-      <c r="B3" s="9" t="n">
-        <v>6406</v>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
-        <is>
-          <t>Максим Яловий Чинадієво</t>
-        </is>
-      </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>Другий платіж</t>
-        </is>
-      </c>
-      <c r="E3" s="11" t="n">
-        <v>218602</v>
-      </c>
-      <c r="F3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="11">
-        <f>E3-F3</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="E4" s="13">
-        <f>SUM(E2:E3)</f>
-        <v/>
-      </c>
-      <c r="F4" s="13">
-        <f>SUM(F2:F3)</f>
-        <v/>
-      </c>
-      <c r="G4" s="13">
-        <f>SUM(G2:G3)</f>
+      <c r="E3" s="13">
+        <f>SUM(E2:E2)</f>
+        <v/>
+      </c>
+      <c r="F3" s="13">
+        <f>SUM(F2:F2)</f>
+        <v/>
+      </c>
+      <c r="G3" s="13">
+        <f>SUM(G2:G2)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G3"/>
+  <autoFilter ref="A1:G2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Іщук update 26.08: 6406 & 8238 cr знято (active), 8238 ризик знято
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -3787,7 +3787,7 @@
     </row>
     <row r="72">
       <c r="A72" s="8" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="B72" s="9" t="n">
         <v>6406</v>
@@ -4947,7 +4947,7 @@
     </row>
     <row r="2">
       <c r="A2" s="8" t="n">
-        <v>46259</v>
+        <v>46260</v>
       </c>
       <c r="B2" s="9" t="n">
         <v>6406</v>

</xml_diff>

<commit_message>
6024 real re-export: cr, risks from file, 78%
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$90</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3275,7 +3275,7 @@
         <v>201600</v>
       </c>
       <c r="G60" s="10" t="n">
-        <v>201600</v>
+        <v>0</v>
       </c>
       <c r="H60" s="11">
         <f>F60-G60</f>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="I60" s="9" t="inlineStr">
         <is>
-          <t>отримано</t>
+          <t>прострочено</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
@@ -4503,7 +4503,7 @@
     </row>
     <row r="88">
       <c r="A88" s="8" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B88" s="9" t="n">
         <v>6024</v>
@@ -4520,7 +4520,7 @@
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>Етап 2</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F88" s="10" t="n">
@@ -4896,7 +4896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4974,26 +4974,54 @@
       </c>
     </row>
     <row r="3">
-      <c r="D3" s="3" t="inlineStr">
+      <c r="A3" s="8" t="n">
+        <v>46237</v>
+      </c>
+      <c r="B3" s="9" t="n">
+        <v>6024</v>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Авансовий платіж</t>
+        </is>
+      </c>
+      <c r="E3" s="11" t="n">
+        <v>201600</v>
+      </c>
+      <c r="F3" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="11">
+        <f>E3-F3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="E3" s="13">
-        <f>SUM(E2:E2)</f>
-        <v/>
-      </c>
-      <c r="F3" s="13">
-        <f>SUM(F2:F2)</f>
-        <v/>
-      </c>
-      <c r="G3" s="13">
-        <f>SUM(G2:G2)</f>
+      <c r="E4" s="13">
+        <f>SUM(E2:E3)</f>
+        <v/>
+      </c>
+      <c r="F4" s="13">
+        <f>SUM(F2:F3)</f>
+        <v/>
+      </c>
+      <c r="G4" s="13">
+        <f>SUM(G2:G3)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G2"/>
+  <autoFilter ref="A1:G3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
+5 нових проєктів (6356,5904,8497,7961,6824) part 1/2 — portfolio+PM+cashflow+hub
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прострочені" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$96</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -519,7 +519,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Дані: 30.08.2026 · без проєктів на паузі/втрачених</t>
+          <t>Дані: 31.08.2026 · без проєктів на паузі/втрачених</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K91"/>
+  <dimension ref="A1:K97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3611,31 +3611,31 @@
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
-        <v>46255</v>
+        <v>46244</v>
       </c>
       <c r="B68" s="9" t="n">
-        <v>7414</v>
+        <v>6824</v>
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ Фундамент домобудування Володимир</t>
+          <t>SOLAR Карпорти 2</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Авансовий платіж</t>
+          <t>Авансовий</t>
         </is>
       </c>
       <c r="F68" s="10" t="n">
-        <v>94000</v>
+        <v>149710</v>
       </c>
       <c r="G68" s="10" t="n">
-        <v>94000</v>
+        <v>149710</v>
       </c>
       <c r="H68" s="11">
         <f>F68-G68</f>
@@ -3655,31 +3655,31 @@
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
-        <v>46255</v>
+        <v>46253</v>
       </c>
       <c r="B69" s="9" t="n">
-        <v>7894</v>
+        <v>5904</v>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>SCP Фора  Хотів</t>
+          <t>SOLAR Карпорти Realcom</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Авансовий</t>
         </is>
       </c>
       <c r="F69" s="10" t="n">
-        <v>185968</v>
+        <v>560757.75</v>
       </c>
       <c r="G69" s="10" t="n">
-        <v>185968</v>
+        <v>560757.75</v>
       </c>
       <c r="H69" s="11">
         <f>F69-G69</f>
@@ -3695,35 +3695,39 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K69" s="12" t="inlineStr"/>
+      <c r="K69" s="12" t="inlineStr">
+        <is>
+          <t>€10 815</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
         <v>46255</v>
       </c>
       <c r="B70" s="9" t="n">
-        <v>7894</v>
+        <v>7414</v>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>SCP Фора  Хотів</t>
+          <t>-26 ГШ Фундамент домобудування Володимир</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F70" s="10" t="n">
-        <v>185967.99</v>
+        <v>94000</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>185967.99</v>
+        <v>94000</v>
       </c>
       <c r="H70" s="11">
         <f>F70-G70</f>
@@ -3760,14 +3764,14 @@
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F71" s="10" t="n">
-        <v>737597.4</v>
+        <v>185968</v>
       </c>
       <c r="G71" s="10" t="n">
-        <v>737597.4</v>
+        <v>185968</v>
       </c>
       <c r="H71" s="11">
         <f>F71-G71</f>
@@ -3790,11 +3794,11 @@
         <v>46255</v>
       </c>
       <c r="B72" s="9" t="n">
-        <v>8898</v>
+        <v>7894</v>
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>Григорівка №3</t>
+          <t>SCP Фора  Хотів</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
@@ -3804,14 +3808,14 @@
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F72" s="10" t="n">
-        <v>188043.75</v>
+        <v>185967.99</v>
       </c>
       <c r="G72" s="10" t="n">
-        <v>188043.75</v>
+        <v>185967.99</v>
       </c>
       <c r="H72" s="11">
         <f>F72-G72</f>
@@ -3831,31 +3835,31 @@
     </row>
     <row r="73">
       <c r="A73" s="8" t="n">
-        <v>46260</v>
+        <v>46255</v>
       </c>
       <c r="B73" s="9" t="n">
-        <v>6406</v>
+        <v>7894</v>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>Максим Яловий Чинадієво</t>
+          <t>SCP Фора  Хотів</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
         <is>
-          <t>Іщук</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F73" s="10" t="n">
-        <v>218602</v>
+        <v>737597.4</v>
       </c>
       <c r="G73" s="10" t="n">
-        <v>170788</v>
+        <v>737597.4</v>
       </c>
       <c r="H73" s="11">
         <f>F73-G73</f>
@@ -3863,7 +3867,7 @@
       </c>
       <c r="I73" s="9" t="inlineStr">
         <is>
-          <t>прострочено</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
@@ -3875,31 +3879,31 @@
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
-        <v>46265</v>
+        <v>46255</v>
       </c>
       <c r="B74" s="9" t="n">
-        <v>8878</v>
+        <v>8898</v>
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
+          <t>Григорівка №3</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F74" s="10" t="n">
-        <v>12823</v>
+        <v>188043.75</v>
       </c>
       <c r="G74" s="10" t="n">
-        <v>12823</v>
+        <v>188043.75</v>
       </c>
       <c r="H74" s="11">
         <f>F74-G74</f>
@@ -3919,31 +3923,31 @@
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
-        <v>46267</v>
+        <v>46260</v>
       </c>
       <c r="B75" s="9" t="n">
-        <v>4766</v>
+        <v>6406</v>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>ALTECO Carport Model Taurus 280кВт</t>
+          <t>Максим Яловий Чинадієво</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Іщук</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F75" s="10" t="n">
-        <v>1263447.42</v>
+        <v>218602</v>
       </c>
       <c r="G75" s="10" t="n">
-        <v>0</v>
+        <v>170788</v>
       </c>
       <c r="H75" s="11">
         <f>F75-G75</f>
@@ -3951,43 +3955,43 @@
       </c>
       <c r="I75" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>прострочено</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-08</t>
         </is>
       </c>
       <c r="K75" s="12" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
-        <v>46269</v>
+        <v>46265</v>
       </c>
       <c r="B76" s="9" t="n">
-        <v>5870</v>
+        <v>8878</v>
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>Carport Airport Munich</t>
+          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Хома</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F76" s="10" t="n">
-        <v>907375</v>
+        <v>12823</v>
       </c>
       <c r="G76" s="10" t="n">
-        <v>0</v>
+        <v>12823</v>
       </c>
       <c r="H76" s="11">
         <f>F76-G76</f>
@@ -3995,47 +3999,43 @@
       </c>
       <c r="I76" s="9" t="inlineStr">
         <is>
-          <t>очікується</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="K76" s="12" t="inlineStr">
-        <is>
-          <t>€17 500</t>
-        </is>
-      </c>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="K76" s="12" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="8" t="n">
-        <v>46270</v>
+        <v>46267</v>
       </c>
       <c r="B77" s="9" t="n">
-        <v>5910</v>
+        <v>4766</v>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>SGM Brdovec, Хорватия</t>
+          <t>ALTECO Carport Model Taurus 280кВт</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E77" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж 60%</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F77" s="10" t="n">
-        <v>17327284.85</v>
+        <v>1263447.42</v>
       </c>
       <c r="G77" s="10" t="n">
-        <v>2977227</v>
+        <v>0</v>
       </c>
       <c r="H77" s="11">
         <f>F77-G77</f>
@@ -4051,36 +4051,32 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="K77" s="12" t="inlineStr">
-        <is>
-          <t>€334 181</t>
-        </is>
-      </c>
+      <c r="K77" s="12" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="8" t="n">
-        <v>46273</v>
+        <v>46269</v>
       </c>
       <c r="B78" s="9" t="n">
-        <v>7002</v>
+        <v>5870</v>
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>Фора SCP Млиново</t>
+          <t>Carport Airport Munich</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E78" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F78" s="10" t="n">
-        <v>573945</v>
+        <v>907375</v>
       </c>
       <c r="G78" s="10" t="n">
         <v>0</v>
@@ -4099,18 +4095,22 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="K78" s="12" t="inlineStr"/>
+      <c r="K78" s="12" t="inlineStr">
+        <is>
+          <t>€17 500</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="8" t="n">
-        <v>46274</v>
+        <v>46270</v>
       </c>
       <c r="B79" s="9" t="n">
-        <v>3456</v>
+        <v>5910</v>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>А Підселання фундаменту</t>
+          <t>SGM Brdovec, Хорватия</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
@@ -4120,14 +4120,14 @@
       </c>
       <c r="E79" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж 60%</t>
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>335974.68</v>
+        <v>17327284.85</v>
       </c>
       <c r="G79" s="10" t="n">
-        <v>0</v>
+        <v>2977227</v>
       </c>
       <c r="H79" s="11">
         <f>F79-G79</f>
@@ -4143,18 +4143,22 @@
           <t>2026-09</t>
         </is>
       </c>
-      <c r="K79" s="12" t="inlineStr"/>
+      <c r="K79" s="12" t="inlineStr">
+        <is>
+          <t>€334 181</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="8" t="n">
-        <v>46280</v>
+        <v>46273</v>
       </c>
       <c r="B80" s="9" t="n">
-        <v>8898</v>
+        <v>7002</v>
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>Григорівка №3</t>
+          <t>Фора SCP Млиново</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
@@ -4164,11 +4168,11 @@
       </c>
       <c r="E80" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F80" s="10" t="n">
-        <v>188043.75</v>
+        <v>573945</v>
       </c>
       <c r="G80" s="10" t="n">
         <v>0</v>
@@ -4191,19 +4195,19 @@
     </row>
     <row r="81">
       <c r="A81" s="8" t="n">
-        <v>46283</v>
+        <v>46274</v>
       </c>
       <c r="B81" s="9" t="n">
-        <v>7508</v>
+        <v>3456</v>
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>8602 Євген Весільна тераса Подорожнє</t>
+          <t>А Підселання фундаменту</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E81" s="9" t="inlineStr">
@@ -4212,7 +4216,7 @@
         </is>
       </c>
       <c r="F81" s="10" t="n">
-        <v>750999.9399999999</v>
+        <v>335974.68</v>
       </c>
       <c r="G81" s="10" t="n">
         <v>0</v>
@@ -4235,28 +4239,28 @@
     </row>
     <row r="82">
       <c r="A82" s="8" t="n">
-        <v>46288</v>
+        <v>46280</v>
       </c>
       <c r="B82" s="9" t="n">
-        <v>7414</v>
+        <v>6356</v>
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ Фундамент домобудування Володимир</t>
+          <t>-26 SOLAR Наземні СЕС Kirill Trokhin</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Авансовий</t>
         </is>
       </c>
       <c r="F82" s="10" t="n">
-        <v>57497.5</v>
+        <v>73128.39999999999</v>
       </c>
       <c r="G82" s="10" t="n">
         <v>0</v>
@@ -4279,28 +4283,28 @@
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
-        <v>46293</v>
+        <v>46280</v>
       </c>
       <c r="B83" s="9" t="n">
-        <v>6352</v>
+        <v>6356</v>
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>АБМК SCP Blade 8PS</t>
+          <t>-26 SOLAR Наземні СЕС Kirill Trokhin</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Авансовий 2</t>
         </is>
       </c>
       <c r="F83" s="10" t="n">
-        <v>1119237.26</v>
+        <v>3064</v>
       </c>
       <c r="G83" s="10" t="n">
         <v>0</v>
@@ -4323,14 +4327,14 @@
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
-        <v>46293</v>
+        <v>46280</v>
       </c>
       <c r="B84" s="9" t="n">
-        <v>6352</v>
+        <v>8898</v>
       </c>
       <c r="C84" s="9" t="inlineStr">
         <is>
-          <t>АБМК SCP Blade 8PS</t>
+          <t>Григорівка №3</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
@@ -4340,11 +4344,11 @@
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F84" s="10" t="n">
-        <v>371982.96</v>
+        <v>188043.75</v>
       </c>
       <c r="G84" s="10" t="n">
         <v>0</v>
@@ -4367,14 +4371,14 @@
     </row>
     <row r="85">
       <c r="A85" s="8" t="n">
-        <v>46295</v>
+        <v>46283</v>
       </c>
       <c r="B85" s="9" t="n">
-        <v>7244</v>
+        <v>7508</v>
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>В Модулекс модульна будівля Чернігів</t>
+          <t>8602 Євген Весільна тераса Подорожнє</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
@@ -4384,11 +4388,11 @@
       </c>
       <c r="E85" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F85" s="10" t="n">
-        <v>132708.6</v>
+        <v>750999.9399999999</v>
       </c>
       <c r="G85" s="10" t="n">
         <v>0</v>
@@ -4411,7 +4415,7 @@
     </row>
     <row r="86">
       <c r="A86" s="8" t="n">
-        <v>46295</v>
+        <v>46288</v>
       </c>
       <c r="B86" s="9" t="n">
         <v>7414</v>
@@ -4428,7 +4432,7 @@
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F86" s="10" t="n">
@@ -4455,14 +4459,14 @@
     </row>
     <row r="87">
       <c r="A87" s="8" t="n">
-        <v>46300</v>
+        <v>46293</v>
       </c>
       <c r="B87" s="9" t="n">
-        <v>5910</v>
+        <v>6352</v>
       </c>
       <c r="C87" s="9" t="inlineStr">
         <is>
-          <t>SGM Brdovec, Хорватия</t>
+          <t>АБМК SCP Blade 8PS</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
@@ -4476,10 +4480,10 @@
         </is>
       </c>
       <c r="F87" s="10" t="n">
-        <v>2887733.9</v>
+        <v>1119237.26</v>
       </c>
       <c r="G87" s="10" t="n">
-        <v>248102.25</v>
+        <v>0</v>
       </c>
       <c r="H87" s="11">
         <f>F87-G87</f>
@@ -4492,39 +4496,35 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="K87" s="12" t="inlineStr">
-        <is>
-          <t>€55 694</t>
-        </is>
-      </c>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K87" s="12" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="8" t="n">
-        <v>46304</v>
+        <v>46293</v>
       </c>
       <c r="B88" s="9" t="n">
-        <v>6024</v>
+        <v>6352</v>
       </c>
       <c r="C88" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
+          <t>АБМК SCP Blade 8PS</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F88" s="10" t="n">
-        <v>246402</v>
+        <v>371982.96</v>
       </c>
       <c r="G88" s="10" t="n">
         <v>0</v>
@@ -4540,26 +4540,26 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="K88" s="12" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="8" t="n">
-        <v>46304</v>
+        <v>46295</v>
       </c>
       <c r="B89" s="9" t="n">
-        <v>7894</v>
+        <v>7244</v>
       </c>
       <c r="C89" s="9" t="inlineStr">
         <is>
-          <t>SCP Фора  Хотів</t>
+          <t>В Модулекс модульна будівля Чернігів</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
@@ -4568,7 +4568,7 @@
         </is>
       </c>
       <c r="F89" s="10" t="n">
-        <v>737597.4</v>
+        <v>132708.6</v>
       </c>
       <c r="G89" s="10" t="n">
         <v>0</v>
@@ -4584,35 +4584,35 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>2026-10</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="K89" s="12" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="8" t="n">
-        <v>46321</v>
+        <v>46295</v>
       </c>
       <c r="B90" s="9" t="n">
-        <v>6352</v>
+        <v>7414</v>
       </c>
       <c r="C90" s="9" t="inlineStr">
         <is>
-          <t>АБМК SCP Blade 8PS</t>
+          <t>-26 ГШ Фундамент домобудування Володимир</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>651792.28</v>
+        <v>57497.5</v>
       </c>
       <c r="G90" s="10" t="n">
         <v>0</v>
@@ -4628,32 +4628,300 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="K90" s="12" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="8" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B91" s="9" t="n">
+        <v>5910</v>
+      </c>
+      <c r="C91" s="9" t="inlineStr">
+        <is>
+          <t>SGM Brdovec, Хорватия</t>
+        </is>
+      </c>
+      <c r="D91" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E91" s="9" t="inlineStr">
+        <is>
+          <t>Третій платіж</t>
+        </is>
+      </c>
+      <c r="F91" s="10" t="n">
+        <v>2887733.9</v>
+      </c>
+      <c r="G91" s="10" t="n">
+        <v>248102.25</v>
+      </c>
+      <c r="H91" s="11">
+        <f>F91-G91</f>
+        <v/>
+      </c>
+      <c r="I91" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
           <t>2026-10</t>
         </is>
       </c>
-      <c r="K90" s="12" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="E91" s="3" t="inlineStr">
+      <c r="K91" s="12" t="inlineStr">
+        <is>
+          <t>€55 694</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B92" s="9" t="n">
+        <v>6024</v>
+      </c>
+      <c r="C92" s="9" t="inlineStr">
+        <is>
+          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
+        </is>
+      </c>
+      <c r="D92" s="9" t="inlineStr">
+        <is>
+          <t>Заянчковський</t>
+        </is>
+      </c>
+      <c r="E92" s="9" t="inlineStr">
+        <is>
+          <t>Другий платіж</t>
+        </is>
+      </c>
+      <c r="F92" s="10" t="n">
+        <v>246402</v>
+      </c>
+      <c r="G92" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" s="11">
+        <f>F92-G92</f>
+        <v/>
+      </c>
+      <c r="I92" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="K92" s="12" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="8" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B93" s="9" t="n">
+        <v>7894</v>
+      </c>
+      <c r="C93" s="9" t="inlineStr">
+        <is>
+          <t>SCP Фора  Хотів</t>
+        </is>
+      </c>
+      <c r="D93" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E93" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F93" s="10" t="n">
+        <v>737597.4</v>
+      </c>
+      <c r="G93" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" s="11">
+        <f>F93-G93</f>
+        <v/>
+      </c>
+      <c r="I93" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="K93" s="12" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B94" s="9" t="n">
+        <v>6356</v>
+      </c>
+      <c r="C94" s="9" t="inlineStr">
+        <is>
+          <t>-26 SOLAR Наземні СЕС Kirill Trokhin</t>
+        </is>
+      </c>
+      <c r="D94" s="9" t="inlineStr">
+        <is>
+          <t>Хома</t>
+        </is>
+      </c>
+      <c r="E94" s="9" t="inlineStr">
+        <is>
+          <t>Етап 2</t>
+        </is>
+      </c>
+      <c r="F94" s="10" t="n">
+        <v>64240</v>
+      </c>
+      <c r="G94" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" s="11">
+        <f>F94-G94</f>
+        <v/>
+      </c>
+      <c r="I94" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="K94" s="12" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="8" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B95" s="9" t="n">
+        <v>6352</v>
+      </c>
+      <c r="C95" s="9" t="inlineStr">
+        <is>
+          <t>АБМК SCP Blade 8PS</t>
+        </is>
+      </c>
+      <c r="D95" s="9" t="inlineStr">
+        <is>
+          <t>Донська</t>
+        </is>
+      </c>
+      <c r="E95" s="9" t="inlineStr">
+        <is>
+          <t>П'ятий платіж</t>
+        </is>
+      </c>
+      <c r="F95" s="10" t="n">
+        <v>651792.28</v>
+      </c>
+      <c r="G95" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" s="11">
+        <f>F95-G95</f>
+        <v/>
+      </c>
+      <c r="I95" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="K95" s="12" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="8" t="n">
+        <v>46331</v>
+      </c>
+      <c r="B96" s="9" t="n">
+        <v>6356</v>
+      </c>
+      <c r="C96" s="9" t="inlineStr">
+        <is>
+          <t>-26 SOLAR Наземні СЕС Kirill Trokhin</t>
+        </is>
+      </c>
+      <c r="D96" s="9" t="inlineStr">
+        <is>
+          <t>Хома</t>
+        </is>
+      </c>
+      <c r="E96" s="9" t="inlineStr">
+        <is>
+          <t>Етап 3</t>
+        </is>
+      </c>
+      <c r="F96" s="10" t="n">
+        <v>12848</v>
+      </c>
+      <c r="G96" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" s="11">
+        <f>F96-G96</f>
+        <v/>
+      </c>
+      <c r="I96" s="9" t="inlineStr">
+        <is>
+          <t>очікується</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>2026-11</t>
+        </is>
+      </c>
+      <c r="K96" s="12" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="E97" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="F91" s="13">
-        <f>SUM(F2:F90)</f>
-        <v/>
-      </c>
-      <c r="G91" s="13">
-        <f>SUM(G2:G90)</f>
-        <v/>
-      </c>
-      <c r="H91" s="13">
-        <f>SUM(H2:H90)</f>
+      <c r="F97" s="13">
+        <f>SUM(F2:F96)</f>
+        <v/>
+      </c>
+      <c r="G97" s="13">
+        <f>SUM(G2:G96)</f>
+        <v/>
+      </c>
+      <c r="H97" s="13">
+        <f>SUM(H2:H96)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I90"/>
+  <autoFilter ref="A1:I96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4664,7 +4932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -4863,25 +5131,48 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>лис 2026</t>
+        </is>
+      </c>
+      <c r="B9" s="11">
+        <f>SUMIF('Графік надходжень'!J:J,"2026-11",'Графік надходжень'!F:F)</f>
+        <v/>
+      </c>
+      <c r="C9" s="11">
+        <f>SUMIF('Графік надходжень'!J:J,"2026-11",'Графік надходжень'!G:G)</f>
+        <v/>
+      </c>
+      <c r="D9" s="11">
+        <f>B9-C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="14">
+        <f>IF(B9=0,0,C9/B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="B9" s="13">
-        <f>SUM(B2:B8)</f>
-        <v/>
-      </c>
-      <c r="C9" s="13">
-        <f>SUM(C2:C8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="13">
-        <f>SUM(D2:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="15">
-        <f>IF(B9=0,0,C9/B9)</f>
+      <c r="B10" s="13">
+        <f>SUM(B2:B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="13">
+        <f>SUM(C2:C9)</f>
+        <v/>
+      </c>
+      <c r="D10" s="13">
+        <f>SUM(D2:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="15">
+        <f>IF(B10=0,0,C10/B10)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 31.08: ПМ 5 нових з Planner, NBU 51.88/44.55 part 1/2
</commit_message>
<xml_diff>
--- a/pillar_cashflow.xlsx
+++ b/pillar_cashflow.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прострочені" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Графік надходжень'!$A$1:$I$94</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Прострочені'!$A$1:$G$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K97"/>
+  <dimension ref="A1:K95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1048,10 +1048,10 @@
         </is>
       </c>
       <c r="F10" s="10" t="n">
-        <v>2592500</v>
+        <v>2594000</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>2592500</v>
+        <v>2594000</v>
       </c>
       <c r="H10" s="11">
         <f>F10-G10</f>
@@ -1096,10 +1096,10 @@
         </is>
       </c>
       <c r="F11" s="10" t="n">
-        <v>5185000</v>
+        <v>5188000</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>5185000</v>
+        <v>5188000</v>
       </c>
       <c r="H11" s="11">
         <f>F11-G11</f>
@@ -2332,10 +2332,10 @@
         </is>
       </c>
       <c r="F39" s="10" t="n">
-        <v>1866600</v>
+        <v>1867680</v>
       </c>
       <c r="G39" s="10" t="n">
-        <v>1866600</v>
+        <v>1867680</v>
       </c>
       <c r="H39" s="11">
         <f>F39-G39</f>
@@ -2556,10 +2556,10 @@
         </is>
       </c>
       <c r="F44" s="10" t="n">
-        <v>456280</v>
+        <v>456544</v>
       </c>
       <c r="G44" s="10" t="n">
-        <v>456280</v>
+        <v>456544</v>
       </c>
       <c r="H44" s="11">
         <f>F44-G44</f>
@@ -3000,10 +3000,10 @@
         </is>
       </c>
       <c r="F54" s="10" t="n">
-        <v>8663616.5</v>
+        <v>8668629.200000001</v>
       </c>
       <c r="G54" s="10" t="n">
-        <v>8663616.5</v>
+        <v>8668629.200000001</v>
       </c>
       <c r="H54" s="11">
         <f>F54-G54</f>
@@ -3136,10 +3136,10 @@
         </is>
       </c>
       <c r="F57" s="10" t="n">
-        <v>4080595</v>
+        <v>4082956</v>
       </c>
       <c r="G57" s="10" t="n">
-        <v>4080595</v>
+        <v>4082956</v>
       </c>
       <c r="H57" s="11">
         <f>F57-G57</f>
@@ -3536,10 +3536,10 @@
         </is>
       </c>
       <c r="F66" s="10" t="n">
-        <v>4963341.25</v>
+        <v>4966213</v>
       </c>
       <c r="G66" s="10" t="n">
-        <v>4963341.25</v>
+        <v>4966213</v>
       </c>
       <c r="H66" s="11">
         <f>F66-G66</f>
@@ -3584,10 +3584,10 @@
         </is>
       </c>
       <c r="F67" s="10" t="n">
-        <v>755713.75</v>
+        <v>756151</v>
       </c>
       <c r="G67" s="10" t="n">
-        <v>755713.75</v>
+        <v>756151</v>
       </c>
       <c r="H67" s="11">
         <f>F67-G67</f>
@@ -3611,14 +3611,14 @@
     </row>
     <row r="68">
       <c r="A68" s="8" t="n">
-        <v>46244</v>
+        <v>46253</v>
       </c>
       <c r="B68" s="9" t="n">
-        <v>6824</v>
+        <v>5904</v>
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>SOLAR Карпорти 2</t>
+          <t>SOLAR Карпорти шт. 10 шт. 0.03 Мвт SIA Realcom</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -3628,14 +3628,14 @@
       </c>
       <c r="E68" s="9" t="inlineStr">
         <is>
-          <t>Авансовий</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F68" s="10" t="n">
-        <v>149710</v>
+        <v>10815</v>
       </c>
       <c r="G68" s="10" t="n">
-        <v>149710</v>
+        <v>10815</v>
       </c>
       <c r="H68" s="11">
         <f>F68-G68</f>
@@ -3655,31 +3655,31 @@
     </row>
     <row r="69">
       <c r="A69" s="8" t="n">
-        <v>46253</v>
+        <v>46255</v>
       </c>
       <c r="B69" s="9" t="n">
-        <v>5904</v>
+        <v>7414</v>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>SOLAR Карпорти Realcom</t>
+          <t>-26 ГШ Фундамент домобудування Володимир</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
         <is>
-          <t>Хома</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E69" s="9" t="inlineStr">
         <is>
-          <t>Авансовий</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F69" s="10" t="n">
-        <v>560757.75</v>
+        <v>94000</v>
       </c>
       <c r="G69" s="10" t="n">
-        <v>560757.75</v>
+        <v>94000</v>
       </c>
       <c r="H69" s="11">
         <f>F69-G69</f>
@@ -3695,39 +3695,35 @@
           <t>2026-08</t>
         </is>
       </c>
-      <c r="K69" s="12" t="inlineStr">
-        <is>
-          <t>€10 815</t>
-        </is>
-      </c>
+      <c r="K69" s="12" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="8" t="n">
         <v>46255</v>
       </c>
       <c r="B70" s="9" t="n">
-        <v>7414</v>
+        <v>7894</v>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ Фундамент домобудування Володимир</t>
+          <t>SCP Фора  Хотів</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E70" s="9" t="inlineStr">
         <is>
-          <t>Авансовий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F70" s="10" t="n">
-        <v>94000</v>
+        <v>185968</v>
       </c>
       <c r="G70" s="10" t="n">
-        <v>94000</v>
+        <v>185968</v>
       </c>
       <c r="H70" s="11">
         <f>F70-G70</f>
@@ -3764,14 +3760,14 @@
       </c>
       <c r="E71" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F71" s="10" t="n">
-        <v>185968</v>
+        <v>185967.99</v>
       </c>
       <c r="G71" s="10" t="n">
-        <v>185968</v>
+        <v>185967.99</v>
       </c>
       <c r="H71" s="11">
         <f>F71-G71</f>
@@ -3808,14 +3804,14 @@
       </c>
       <c r="E72" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F72" s="10" t="n">
-        <v>185967.99</v>
+        <v>737597.4</v>
       </c>
       <c r="G72" s="10" t="n">
-        <v>185967.99</v>
+        <v>737597.4</v>
       </c>
       <c r="H72" s="11">
         <f>F72-G72</f>
@@ -3838,11 +3834,11 @@
         <v>46255</v>
       </c>
       <c r="B73" s="9" t="n">
-        <v>7894</v>
+        <v>8898</v>
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>SCP Фора  Хотів</t>
+          <t>Григорівка №3</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
@@ -3852,14 +3848,14 @@
       </c>
       <c r="E73" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F73" s="10" t="n">
-        <v>737597.4</v>
+        <v>188043.75</v>
       </c>
       <c r="G73" s="10" t="n">
-        <v>737597.4</v>
+        <v>188043.75</v>
       </c>
       <c r="H73" s="11">
         <f>F73-G73</f>
@@ -3879,19 +3875,19 @@
     </row>
     <row r="74">
       <c r="A74" s="8" t="n">
-        <v>46255</v>
+        <v>46260</v>
       </c>
       <c r="B74" s="9" t="n">
-        <v>8898</v>
+        <v>6406</v>
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>Григорівка №3</t>
+          <t>Максим Яловий Чинадієво</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Іщук</t>
         </is>
       </c>
       <c r="E74" s="9" t="inlineStr">
@@ -3900,10 +3896,10 @@
         </is>
       </c>
       <c r="F74" s="10" t="n">
-        <v>188043.75</v>
+        <v>218602</v>
       </c>
       <c r="G74" s="10" t="n">
-        <v>188043.75</v>
+        <v>170788</v>
       </c>
       <c r="H74" s="11">
         <f>F74-G74</f>
@@ -3911,7 +3907,7 @@
       </c>
       <c r="I74" s="9" t="inlineStr">
         <is>
-          <t>отримано</t>
+          <t>прострочено</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
@@ -3923,31 +3919,31 @@
     </row>
     <row r="75">
       <c r="A75" s="8" t="n">
-        <v>46260</v>
+        <v>46265</v>
       </c>
       <c r="B75" s="9" t="n">
-        <v>6406</v>
+        <v>8878</v>
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>Максим Яловий Чинадієво</t>
+          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
         <is>
-          <t>Іщук</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E75" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F75" s="10" t="n">
-        <v>218602</v>
+        <v>12823</v>
       </c>
       <c r="G75" s="10" t="n">
-        <v>170788</v>
+        <v>12823</v>
       </c>
       <c r="H75" s="11">
         <f>F75-G75</f>
@@ -3955,7 +3951,7 @@
       </c>
       <c r="I75" s="9" t="inlineStr">
         <is>
-          <t>прострочено</t>
+          <t>отримано</t>
         </is>
       </c>
       <c r="J75" t="inlineStr">
@@ -3967,31 +3963,31 @@
     </row>
     <row r="76">
       <c r="A76" s="8" t="n">
-        <v>46265</v>
+        <v>46266</v>
       </c>
       <c r="B76" s="9" t="n">
-        <v>8878</v>
+        <v>6356</v>
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>А ТОВ КОМПАНІЯ ВОЛЬТ СЕРВІС ГРУП</t>
+          <t>-26 SOLAR Наземні СЕС 3 Kirill Trokhin</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E76" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Авансовий платіж</t>
         </is>
       </c>
       <c r="F76" s="10" t="n">
-        <v>12823</v>
+        <v>51392</v>
       </c>
       <c r="G76" s="10" t="n">
-        <v>12823</v>
+        <v>0</v>
       </c>
       <c r="H76" s="11">
         <f>F76-G76</f>
@@ -3999,12 +3995,12 @@
       </c>
       <c r="I76" s="9" t="inlineStr">
         <is>
-          <t>отримано</t>
+          <t>очікується</t>
         </is>
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-09</t>
         </is>
       </c>
       <c r="K76" s="12" t="inlineStr"/>
@@ -4076,7 +4072,7 @@
         </is>
       </c>
       <c r="F78" s="10" t="n">
-        <v>907375</v>
+        <v>907900</v>
       </c>
       <c r="G78" s="10" t="n">
         <v>0</v>
@@ -4124,10 +4120,10 @@
         </is>
       </c>
       <c r="F79" s="10" t="n">
-        <v>17327284.85</v>
+        <v>17337310.28</v>
       </c>
       <c r="G79" s="10" t="n">
-        <v>2977227</v>
+        <v>2978949.6</v>
       </c>
       <c r="H79" s="11">
         <f>F79-G79</f>
@@ -4242,25 +4238,25 @@
         <v>46280</v>
       </c>
       <c r="B82" s="9" t="n">
-        <v>6356</v>
+        <v>8898</v>
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>-26 SOLAR Наземні СЕС Kirill Trokhin</t>
+          <t>Григорівка №3</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
         <is>
-          <t>Хома</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E82" s="9" t="inlineStr">
         <is>
-          <t>Авансовий</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F82" s="10" t="n">
-        <v>73128.39999999999</v>
+        <v>188043.75</v>
       </c>
       <c r="G82" s="10" t="n">
         <v>0</v>
@@ -4283,28 +4279,28 @@
     </row>
     <row r="83">
       <c r="A83" s="8" t="n">
-        <v>46280</v>
+        <v>46283</v>
       </c>
       <c r="B83" s="9" t="n">
-        <v>6356</v>
+        <v>7508</v>
       </c>
       <c r="C83" s="9" t="inlineStr">
         <is>
-          <t>-26 SOLAR Наземні СЕС Kirill Trokhin</t>
+          <t>8602 Євген Весільна тераса Подорожнє</t>
         </is>
       </c>
       <c r="D83" s="9" t="inlineStr">
         <is>
-          <t>Хома</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E83" s="9" t="inlineStr">
         <is>
-          <t>Авансовий 2</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F83" s="10" t="n">
-        <v>3064</v>
+        <v>750999.9399999999</v>
       </c>
       <c r="G83" s="10" t="n">
         <v>0</v>
@@ -4327,28 +4323,28 @@
     </row>
     <row r="84">
       <c r="A84" s="8" t="n">
-        <v>46280</v>
+        <v>46288</v>
       </c>
       <c r="B84" s="9" t="n">
-        <v>8898</v>
+        <v>7414</v>
       </c>
       <c r="C84" s="9" t="inlineStr">
         <is>
-          <t>Григорівка №3</t>
+          <t>-26 ГШ Фундамент домобудування Володимир</t>
         </is>
       </c>
       <c r="D84" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E84" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F84" s="10" t="n">
-        <v>188043.75</v>
+        <v>57497.5</v>
       </c>
       <c r="G84" s="10" t="n">
         <v>0</v>
@@ -4371,19 +4367,19 @@
     </row>
     <row r="85">
       <c r="A85" s="8" t="n">
-        <v>46283</v>
+        <v>46293</v>
       </c>
       <c r="B85" s="9" t="n">
-        <v>7508</v>
+        <v>6352</v>
       </c>
       <c r="C85" s="9" t="inlineStr">
         <is>
-          <t>8602 Євген Весільна тераса Подорожнє</t>
+          <t>АБМК SCP Blade 8PS</t>
         </is>
       </c>
       <c r="D85" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E85" s="9" t="inlineStr">
@@ -4392,7 +4388,7 @@
         </is>
       </c>
       <c r="F85" s="10" t="n">
-        <v>750999.9399999999</v>
+        <v>1119237.26</v>
       </c>
       <c r="G85" s="10" t="n">
         <v>0</v>
@@ -4415,28 +4411,28 @@
     </row>
     <row r="86">
       <c r="A86" s="8" t="n">
-        <v>46288</v>
+        <v>46293</v>
       </c>
       <c r="B86" s="9" t="n">
-        <v>7414</v>
+        <v>6352</v>
       </c>
       <c r="C86" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ Фундамент домобудування Володимир</t>
+          <t>АБМК SCP Blade 8PS</t>
         </is>
       </c>
       <c r="D86" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E86" s="9" t="inlineStr">
         <is>
-          <t>Другий платіж</t>
+          <t>Четвертий платіж</t>
         </is>
       </c>
       <c r="F86" s="10" t="n">
-        <v>57497.5</v>
+        <v>371982.96</v>
       </c>
       <c r="G86" s="10" t="n">
         <v>0</v>
@@ -4459,28 +4455,28 @@
     </row>
     <row r="87">
       <c r="A87" s="8" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="B87" s="9" t="n">
-        <v>6352</v>
+        <v>7244</v>
       </c>
       <c r="C87" s="9" t="inlineStr">
         <is>
-          <t>АБМК SCP Blade 8PS</t>
+          <t>В Модулекс модульна будівля Чернігів</t>
         </is>
       </c>
       <c r="D87" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E87" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F87" s="10" t="n">
-        <v>1119237.26</v>
+        <v>132708.6</v>
       </c>
       <c r="G87" s="10" t="n">
         <v>0</v>
@@ -4503,28 +4499,28 @@
     </row>
     <row r="88">
       <c r="A88" s="8" t="n">
-        <v>46293</v>
+        <v>46295</v>
       </c>
       <c r="B88" s="9" t="n">
-        <v>6352</v>
+        <v>7414</v>
       </c>
       <c r="C88" s="9" t="inlineStr">
         <is>
-          <t>АБМК SCP Blade 8PS</t>
+          <t>-26 ГШ Фундамент домобудування Володимир</t>
         </is>
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Донська</t>
+          <t>Заянчковський</t>
         </is>
       </c>
       <c r="E88" s="9" t="inlineStr">
         <is>
-          <t>Четвертий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F88" s="10" t="n">
-        <v>371982.96</v>
+        <v>57497.5</v>
       </c>
       <c r="G88" s="10" t="n">
         <v>0</v>
@@ -4547,31 +4543,31 @@
     </row>
     <row r="89">
       <c r="A89" s="8" t="n">
-        <v>46295</v>
+        <v>46300</v>
       </c>
       <c r="B89" s="9" t="n">
-        <v>7244</v>
+        <v>5910</v>
       </c>
       <c r="C89" s="9" t="inlineStr">
         <is>
-          <t>В Модулекс модульна будівля Чернігів</t>
+          <t>SGM Brdovec, Хорватия</t>
         </is>
       </c>
       <c r="D89" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Донська</t>
         </is>
       </c>
       <c r="E89" s="9" t="inlineStr">
         <is>
-          <t>П'ятий платіж</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F89" s="10" t="n">
-        <v>132708.6</v>
+        <v>2889404.72</v>
       </c>
       <c r="G89" s="10" t="n">
-        <v>0</v>
+        <v>248245.8</v>
       </c>
       <c r="H89" s="11">
         <f>F89-G89</f>
@@ -4584,21 +4580,25 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="K89" s="12" t="inlineStr"/>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="K89" s="12" t="inlineStr">
+        <is>
+          <t>€55 694</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="8" t="n">
-        <v>46295</v>
+        <v>46304</v>
       </c>
       <c r="B90" s="9" t="n">
-        <v>7414</v>
+        <v>6024</v>
       </c>
       <c r="C90" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ Фундамент домобудування Володимир</t>
+          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
         </is>
       </c>
       <c r="D90" s="9" t="inlineStr">
@@ -4608,11 +4608,11 @@
       </c>
       <c r="E90" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>Другий платіж</t>
         </is>
       </c>
       <c r="F90" s="10" t="n">
-        <v>57497.5</v>
+        <v>246402</v>
       </c>
       <c r="G90" s="10" t="n">
         <v>0</v>
@@ -4628,21 +4628,21 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>2026-09</t>
+          <t>2026-10</t>
         </is>
       </c>
       <c r="K90" s="12" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="8" t="n">
-        <v>46300</v>
+        <v>46304</v>
       </c>
       <c r="B91" s="9" t="n">
-        <v>5910</v>
+        <v>7894</v>
       </c>
       <c r="C91" s="9" t="inlineStr">
         <is>
-          <t>SGM Brdovec, Хорватия</t>
+          <t>SCP Фора  Хотів</t>
         </is>
       </c>
       <c r="D91" s="9" t="inlineStr">
@@ -4652,14 +4652,14 @@
       </c>
       <c r="E91" s="9" t="inlineStr">
         <is>
-          <t>Третій платіж</t>
+          <t>П'ятий платіж</t>
         </is>
       </c>
       <c r="F91" s="10" t="n">
-        <v>2887733.9</v>
+        <v>737597.4</v>
       </c>
       <c r="G91" s="10" t="n">
-        <v>248102.25</v>
+        <v>0</v>
       </c>
       <c r="H91" s="11">
         <f>F91-G91</f>
@@ -4675,27 +4675,23 @@
           <t>2026-10</t>
         </is>
       </c>
-      <c r="K91" s="12" t="inlineStr">
-        <is>
-          <t>€55 694</t>
-        </is>
-      </c>
+      <c r="K91" s="12" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="8" t="n">
-        <v>46304</v>
+        <v>46316</v>
       </c>
       <c r="B92" s="9" t="n">
-        <v>6024</v>
+        <v>6356</v>
       </c>
       <c r="C92" s="9" t="inlineStr">
         <is>
-          <t>-26 ГШ с. Липовиця Черніг. обл. Модулекс</t>
+          <t>-26 SOLAR Наземні СЕС 3 Kirill Trokhin</t>
         </is>
       </c>
       <c r="D92" s="9" t="inlineStr">
         <is>
-          <t>Заянчковський</t>
+          <t>Хома</t>
         </is>
       </c>
       <c r="E92" s="9" t="inlineStr">
@@ -4704,7 +4700,7 @@
         </is>
       </c>
       <c r="F92" s="10" t="n">
-        <v>246402</v>
+        <v>64240</v>
       </c>
       <c r="G92" s="10" t="n">
         <v>0</v>
@@ -4727,14 +4723,14 @@
     </row>
     <row r="93">
       <c r="A93" s="8" t="n">
-        <v>46304</v>
+        <v>46321</v>
       </c>
       <c r="B93" s="9" t="n">
-        <v>7894</v>
+        <v>6352</v>
       </c>
       <c r="C93" s="9" t="inlineStr">
         <is>
-          <t>SCP Фора  Хотів</t>
+          <t>АБМК SCP Blade 8PS</t>
         </is>
       </c>
       <c r="D93" s="9" t="inlineStr">
@@ -4748,7 +4744,7 @@
         </is>
       </c>
       <c r="F93" s="10" t="n">
-        <v>737597.4</v>
+        <v>651792.28</v>
       </c>
       <c r="G93" s="10" t="n">
         <v>0</v>
@@ -4771,14 +4767,14 @@
     </row>
     <row r="94">
       <c r="A94" s="8" t="n">
-        <v>46310</v>
+        <v>46322</v>
       </c>
       <c r="B94" s="9" t="n">
         <v>6356</v>
       </c>
       <c r="C94" s="9" t="inlineStr">
         <is>
-          <t>-26 SOLAR Наземні СЕС Kirill Trokhin</t>
+          <t>-26 SOLAR Наземні СЕС 3 Kirill Trokhin</t>
         </is>
       </c>
       <c r="D94" s="9" t="inlineStr">
@@ -4788,11 +4784,11 @@
       </c>
       <c r="E94" s="9" t="inlineStr">
         <is>
-          <t>Етап 2</t>
+          <t>Третій платіж</t>
         </is>
       </c>
       <c r="F94" s="10" t="n">
-        <v>64240</v>
+        <v>12848</v>
       </c>
       <c r="G94" s="10" t="n">
         <v>0</v>
@@ -4814,114 +4810,26 @@
       <c r="K94" s="12" t="inlineStr"/>
     </row>
     <row r="95">
-      <c r="A95" s="8" t="n">
-        <v>46321</v>
-      </c>
-      <c r="B95" s="9" t="n">
-        <v>6352</v>
-      </c>
-      <c r="C95" s="9" t="inlineStr">
-        <is>
-          <t>АБМК SCP Blade 8PS</t>
-        </is>
-      </c>
-      <c r="D95" s="9" t="inlineStr">
-        <is>
-          <t>Донська</t>
-        </is>
-      </c>
-      <c r="E95" s="9" t="inlineStr">
-        <is>
-          <t>П'ятий платіж</t>
-        </is>
-      </c>
-      <c r="F95" s="10" t="n">
-        <v>651792.28</v>
-      </c>
-      <c r="G95" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H95" s="11">
-        <f>F95-G95</f>
-        <v/>
-      </c>
-      <c r="I95" s="9" t="inlineStr">
-        <is>
-          <t>очікується</t>
-        </is>
-      </c>
-      <c r="J95" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="K95" s="12" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="8" t="n">
-        <v>46331</v>
-      </c>
-      <c r="B96" s="9" t="n">
-        <v>6356</v>
-      </c>
-      <c r="C96" s="9" t="inlineStr">
-        <is>
-          <t>-26 SOLAR Наземні СЕС Kirill Trokhin</t>
-        </is>
-      </c>
-      <c r="D96" s="9" t="inlineStr">
-        <is>
-          <t>Хома</t>
-        </is>
-      </c>
-      <c r="E96" s="9" t="inlineStr">
-        <is>
-          <t>Етап 3</t>
-        </is>
-      </c>
-      <c r="F96" s="10" t="n">
-        <v>12848</v>
-      </c>
-      <c r="G96" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H96" s="11">
-        <f>F96-G96</f>
-        <v/>
-      </c>
-      <c r="I96" s="9" t="inlineStr">
-        <is>
-          <t>очікується</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr">
-        <is>
-          <t>2026-11</t>
-        </is>
-      </c>
-      <c r="K96" s="12" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="E97" s="3" t="inlineStr">
+      <c r="E95" s="3" t="inlineStr">
         <is>
           <t>Разом</t>
         </is>
       </c>
-      <c r="F97" s="13">
-        <f>SUM(F2:F96)</f>
-        <v/>
-      </c>
-      <c r="G97" s="13">
-        <f>SUM(G2:G96)</f>
-        <v/>
-      </c>
-      <c r="H97" s="13">
-        <f>SUM(H2:H96)</f>
+      <c r="F95" s="13">
+        <f>SUM(F2:F94)</f>
+        <v/>
+      </c>
+      <c r="G95" s="13">
+        <f>SUM(G2:G94)</f>
+        <v/>
+      </c>
+      <c r="H95" s="13">
+        <f>SUM(H2:H94)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I96"/>
+  <autoFilter ref="A1:I94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4932,7 +4840,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5131,48 +5039,25 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="inlineStr">
-        <is>
-          <t>лис 2026</t>
-        </is>
-      </c>
-      <c r="B9" s="11">
-        <f>SUMIF('Графік надходжень'!J:J,"2026-11",'Графік надходжень'!F:F)</f>
-        <v/>
-      </c>
-      <c r="C9" s="11">
-        <f>SUMIF('Графік надходжень'!J:J,"2026-11",'Графік надходжень'!G:G)</f>
-        <v/>
-      </c>
-      <c r="D9" s="11">
-        <f>B9-C9</f>
-        <v/>
-      </c>
-      <c r="E9" s="14">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Разом</t>
+        </is>
+      </c>
+      <c r="B9" s="13">
+        <f>SUM(B2:B8)</f>
+        <v/>
+      </c>
+      <c r="C9" s="13">
+        <f>SUM(C2:C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="13">
+        <f>SUM(D2:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="15">
         <f>IF(B9=0,0,C9/B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>Разом</t>
-        </is>
-      </c>
-      <c r="B10" s="13">
-        <f>SUM(B2:B9)</f>
-        <v/>
-      </c>
-      <c r="C10" s="13">
-        <f>SUM(C2:C9)</f>
-        <v/>
-      </c>
-      <c r="D10" s="13">
-        <f>SUM(D2:D9)</f>
-        <v/>
-      </c>
-      <c r="E10" s="15">
-        <f>IF(B10=0,0,C10/B10)</f>
         <v/>
       </c>
     </row>

</xml_diff>